<commit_message>
Add 19 sales tools: 4 CRM additions plus new AI Sales Outreach & Prospecting category
https://claude.ai/code/session_01G7pVVMWXdJQpTNJYEckRF2
</commit_message>
<xml_diff>
--- a/AI-Tools-Directory.xlsx
+++ b/AI-Tools-Directory.xlsx
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O215"/>
+  <dimension ref="A1:O235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -12242,62 +12242,62 @@
     </row>
     <row r="190" ht="58" customHeight="1">
       <c r="A190" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=apollo.io&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=salesforce.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B190" s="6" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Salesforce (Agentforce)</t>
         </is>
       </c>
       <c r="C190" s="7" t="inlineStr">
         <is>
-          <t>Freemium</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="D190" s="8" t="inlineStr">
         <is>
-          <t>apollo.io</t>
+          <t>salesforce.com</t>
         </is>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>B2B contact database + sequencing + AI sales engagement</t>
+          <t>Enterprise CRM leader with Agentforce AI agents and Einstein AI</t>
         </is>
       </c>
       <c r="F190" s="7" t="inlineStr">
         <is>
-          <t>Free; from $49/user/mo</t>
+          <t>From $25/user/mo; Agentforce usage-priced extra</t>
         </is>
       </c>
       <c r="G190" s="7" t="inlineStr">
         <is>
-          <t>Partial — API/Zapier; community MCP</t>
+          <t>Yes — Claude available in Agentforce via the Anthropic partnership</t>
         </is>
       </c>
       <c r="H190" s="7" t="inlineStr">
         <is>
-          <t>275M-contact database with outreach in one</t>
+          <t>Enterprise standard; AI agents on your own CRM data</t>
         </is>
       </c>
       <c r="I190" s="7" t="inlineStr">
         <is>
-          <t>Data accuracy varies; email deliverability care</t>
+          <t>Cost and complexity stack quickly</t>
         </is>
       </c>
       <c r="J190" s="7" t="inlineStr">
         <is>
-          <t>Outbound SDR teams</t>
+          <t>Mid-size to enterprise sales orgs</t>
         </is>
       </c>
       <c r="K190" s="5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L190" s="5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M190" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N190" s="5" t="n">
         <v>7.3</v>
@@ -12308,62 +12308,62 @@
     </row>
     <row r="191" ht="58" customHeight="1">
       <c r="A191" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=clay.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=apollo.io&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B191" s="6" t="inlineStr">
         <is>
-          <t>Clay</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="C191" s="7" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Freemium</t>
         </is>
       </c>
       <c r="D191" s="8" t="inlineStr">
         <is>
-          <t>clay.com</t>
+          <t>apollo.io</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>Data enrichment + AI research agent (Claygent) for hyper-personalised outbound</t>
+          <t>B2B contact database + sequencing + AI sales engagement</t>
         </is>
       </c>
       <c r="F191" s="7" t="inlineStr">
         <is>
-          <t>From $134/mo</t>
+          <t>Free; from $49/user/mo</t>
         </is>
       </c>
       <c r="G191" s="7" t="inlineStr">
         <is>
-          <t>Yes — Claude usable as enrichment model</t>
+          <t>Partial — API/Zapier; community MCP</t>
         </is>
       </c>
       <c r="H191" s="7" t="inlineStr">
         <is>
-          <t>Combines 100+ data sources; AI personalisation at scale</t>
+          <t>275M-contact database with outreach in one</t>
         </is>
       </c>
       <c r="I191" s="7" t="inlineStr">
         <is>
-          <t>Steep learning curve and price</t>
+          <t>Data accuracy varies; email deliverability care</t>
         </is>
       </c>
       <c r="J191" s="7" t="inlineStr">
         <is>
-          <t>Growth teams doing serious outbound</t>
+          <t>Outbound SDR teams</t>
         </is>
       </c>
       <c r="K191" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="L191" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="M191" s="5" t="n">
         <v>8</v>
-      </c>
-      <c r="L191" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="M191" s="5" t="n">
-        <v>9</v>
       </c>
       <c r="N191" s="5" t="n">
         <v>7.3</v>
@@ -12374,12 +12374,12 @@
     </row>
     <row r="192" ht="58" customHeight="1">
       <c r="A192" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=gong.io&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=clay.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B192" s="6" t="inlineStr">
         <is>
-          <t>Gong</t>
+          <t>Clay</t>
         </is>
       </c>
       <c r="C192" s="7" t="inlineStr">
@@ -12389,83 +12389,83 @@
       </c>
       <c r="D192" s="8" t="inlineStr">
         <is>
-          <t>gong.io</t>
+          <t>clay.com</t>
         </is>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>Revenue intelligence: call recording, deal insights, forecasting</t>
+          <t>Data enrichment + AI research agent (Claygent) for hyper-personalised outbound</t>
         </is>
       </c>
       <c r="F192" s="7" t="inlineStr">
         <is>
-          <t>~$1,400/user/yr + platform fee</t>
+          <t>From $134/mo</t>
         </is>
       </c>
       <c r="G192" s="7" t="inlineStr">
         <is>
-          <t>Partial — API; Anthropic models used internally</t>
+          <t>Yes — Claude usable as enrichment model</t>
         </is>
       </c>
       <c r="H192" s="7" t="inlineStr">
         <is>
-          <t>Category leader; coaching gold</t>
+          <t>Combines 100+ data sources; AI personalisation at scale</t>
         </is>
       </c>
       <c r="I192" s="7" t="inlineStr">
         <is>
-          <t>Enterprise pricing; adoption effort</t>
+          <t>Steep learning curve and price</t>
         </is>
       </c>
       <c r="J192" s="7" t="inlineStr">
         <is>
-          <t>Sales orgs 20+ reps</t>
+          <t>Growth teams doing serious outbound</t>
         </is>
       </c>
       <c r="K192" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L192" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M192" s="5" t="n">
         <v>9</v>
       </c>
       <c r="N192" s="5" t="n">
-        <v>6.3</v>
+        <v>7.3</v>
       </c>
       <c r="O192" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="193" ht="58" customHeight="1">
       <c r="A193" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=lavender.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=pipedrive.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B193" s="6" t="inlineStr">
         <is>
-          <t>Lavender</t>
+          <t>Pipedrive</t>
         </is>
       </c>
       <c r="C193" s="7" t="inlineStr">
         <is>
-          <t>Freemium</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="D193" s="8" t="inlineStr">
         <is>
-          <t>lavender.ai</t>
+          <t>pipedrive.com</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>AI email coach that scores and improves sales emails</t>
+          <t>Easy SMB sales CRM with AI sales assistant and automations</t>
         </is>
       </c>
       <c r="F193" s="7" t="inlineStr">
         <is>
-          <t>Free; from $27/mo</t>
+          <t>From $14/user/mo</t>
         </is>
       </c>
       <c r="G193" s="7" t="inlineStr">
@@ -12475,43 +12475,43 @@
       </c>
       <c r="H193" s="7" t="inlineStr">
         <is>
-          <t>Real-time coaching improves reply rates</t>
+          <t>Fast to adopt; great pipeline view; fair price</t>
         </is>
       </c>
       <c r="I193" s="7" t="inlineStr">
         <is>
-          <t>Email-only scope</t>
+          <t>Light for complex enterprise needs</t>
         </is>
       </c>
       <c r="J193" s="7" t="inlineStr">
         <is>
-          <t>SDRs writing cold email</t>
+          <t>SMB sales teams</t>
         </is>
       </c>
       <c r="K193" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L193" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M193" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N193" s="5" t="n">
-        <v>5.3</v>
+        <v>6.7</v>
       </c>
       <c r="O193" s="5" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="194" ht="58" customHeight="1">
       <c r="A194" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=outreach.io&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=gong.io&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B194" s="6" t="inlineStr">
         <is>
-          <t>Outreach</t>
+          <t>Gong</t>
         </is>
       </c>
       <c r="C194" s="7" t="inlineStr">
@@ -12521,50 +12521,50 @@
       </c>
       <c r="D194" s="8" t="inlineStr">
         <is>
-          <t>outreach.io</t>
+          <t>gong.io</t>
         </is>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>Enterprise sales engagement and execution platform</t>
+          <t>Revenue intelligence: call recording, deal insights, forecasting</t>
         </is>
       </c>
       <c r="F194" s="7" t="inlineStr">
         <is>
-          <t>~$100+/user/mo</t>
+          <t>~$1,400/user/yr + platform fee</t>
         </is>
       </c>
       <c r="G194" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partial — API; Anthropic models used internally</t>
         </is>
       </c>
       <c r="H194" s="7" t="inlineStr">
         <is>
-          <t>Deep workflows, forecasting; enterprise-grade</t>
+          <t>Category leader; coaching gold</t>
         </is>
       </c>
       <c r="I194" s="7" t="inlineStr">
         <is>
-          <t>Cost &amp; complexity</t>
+          <t>Enterprise pricing; adoption effort</t>
         </is>
       </c>
       <c r="J194" s="7" t="inlineStr">
         <is>
-          <t>Enterprise sales orgs</t>
+          <t>Sales orgs 20+ reps</t>
         </is>
       </c>
       <c r="K194" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L194" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M194" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N194" s="5" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="O194" s="5" t="n">
         <v>8</v>
@@ -12572,12 +12572,12 @@
     </row>
     <row r="195" ht="58" customHeight="1">
       <c r="A195" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=sybill.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=clari.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B195" s="6" t="inlineStr">
         <is>
-          <t>Sybill</t>
+          <t>Clari</t>
         </is>
       </c>
       <c r="C195" s="7" t="inlineStr">
@@ -12587,17 +12587,17 @@
       </c>
       <c r="D195" s="8" t="inlineStr">
         <is>
-          <t>sybill.ai</t>
+          <t>clari.com</t>
         </is>
       </c>
       <c r="E195" s="7" t="inlineStr">
         <is>
-          <t>AI deal copilot: call summaries, CRM autofill, behaviour signals</t>
+          <t>Revenue platform: AI forecasting, deal inspection, pipeline health</t>
         </is>
       </c>
       <c r="F195" s="7" t="inlineStr">
         <is>
-          <t>From $49/user/mo</t>
+          <t>Enterprise custom pricing</t>
         </is>
       </c>
       <c r="G195" s="7" t="inlineStr">
@@ -12607,512 +12607,512 @@
       </c>
       <c r="H195" s="7" t="inlineStr">
         <is>
-          <t>Automatic CRM hygiene; emotion/engagement signals</t>
+          <t>Best-in-class forecasting accuracy</t>
         </is>
       </c>
       <c r="I195" s="7" t="inlineStr">
         <is>
-          <t>Per-seat cost; niche</t>
+          <t>Enterprise price; needs clean CRM data</t>
         </is>
       </c>
       <c r="J195" s="7" t="inlineStr">
         <is>
-          <t>AEs hating CRM data entry</t>
+          <t>Revenue leaders at 50+ rep orgs</t>
         </is>
       </c>
       <c r="K195" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L195" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M195" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N195" s="5" t="n">
         <v>5.7</v>
       </c>
       <c r="O195" s="5" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="196" ht="58" customHeight="1">
+      <c r="A196" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=attention.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B196" s="6" t="inlineStr">
+        <is>
+          <t>Attention</t>
+        </is>
+      </c>
+      <c r="C196" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D196" s="8" t="inlineStr">
+        <is>
+          <t>attention.com</t>
+        </is>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>AI sales assistant: call recording, auto CRM fill, coaching, follow-up emails</t>
+        </is>
+      </c>
+      <c r="F196" s="7" t="inlineStr">
+        <is>
+          <t>From ~$50/user/mo (custom)</t>
+        </is>
+      </c>
+      <c r="G196" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H196" s="7" t="inlineStr">
+        <is>
+          <t>Strong CRM-hygiene automation; fast follow-ups</t>
+        </is>
+      </c>
+      <c r="I196" s="7" t="inlineStr">
+        <is>
+          <t>Younger than Gong; custom pricing</t>
+        </is>
+      </c>
+      <c r="J196" s="7" t="inlineStr">
+        <is>
+          <t>Mid-market sales teams</t>
+        </is>
+      </c>
+      <c r="K196" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L196" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="M196" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N196" s="5" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="O196" s="5" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="197" ht="58" customHeight="1">
+      <c r="A197" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=lavender.ai&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B197" s="6" t="inlineStr">
+        <is>
+          <t>Lavender</t>
+        </is>
+      </c>
+      <c r="C197" s="7" t="inlineStr">
+        <is>
+          <t>Freemium</t>
+        </is>
+      </c>
+      <c r="D197" s="8" t="inlineStr">
+        <is>
+          <t>lavender.ai</t>
+        </is>
+      </c>
+      <c r="E197" s="7" t="inlineStr">
+        <is>
+          <t>AI email coach that scores and improves sales emails</t>
+        </is>
+      </c>
+      <c r="F197" s="7" t="inlineStr">
+        <is>
+          <t>Free; from $27/mo</t>
+        </is>
+      </c>
+      <c r="G197" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H197" s="7" t="inlineStr">
+        <is>
+          <t>Real-time coaching improves reply rates</t>
+        </is>
+      </c>
+      <c r="I197" s="7" t="inlineStr">
+        <is>
+          <t>Email-only scope</t>
+        </is>
+      </c>
+      <c r="J197" s="7" t="inlineStr">
+        <is>
+          <t>SDRs writing cold email</t>
+        </is>
+      </c>
+      <c r="K197" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L197" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M197" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N197" s="5" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="O197" s="5" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="198" ht="58" customHeight="1">
+      <c r="A198" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=outreach.io&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B198" s="6" t="inlineStr">
+        <is>
+          <t>Outreach</t>
+        </is>
+      </c>
+      <c r="C198" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D198" s="8" t="inlineStr">
+        <is>
+          <t>outreach.io</t>
+        </is>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>Enterprise sales engagement and execution platform</t>
+        </is>
+      </c>
+      <c r="F198" s="7" t="inlineStr">
+        <is>
+          <t>~$100+/user/mo</t>
+        </is>
+      </c>
+      <c r="G198" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H198" s="7" t="inlineStr">
+        <is>
+          <t>Deep workflows, forecasting; enterprise-grade</t>
+        </is>
+      </c>
+      <c r="I198" s="7" t="inlineStr">
+        <is>
+          <t>Cost &amp; complexity</t>
+        </is>
+      </c>
+      <c r="J198" s="7" t="inlineStr">
+        <is>
+          <t>Enterprise sales orgs</t>
+        </is>
+      </c>
+      <c r="K198" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L198" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M198" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="N198" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="O198" s="5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="199" ht="58" customHeight="1">
+      <c r="A199" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=sybill.ai&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B199" s="6" t="inlineStr">
+        <is>
+          <t>Sybill</t>
+        </is>
+      </c>
+      <c r="C199" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D199" s="8" t="inlineStr">
+        <is>
+          <t>sybill.ai</t>
+        </is>
+      </c>
+      <c r="E199" s="7" t="inlineStr">
+        <is>
+          <t>AI deal copilot: call summaries, CRM autofill, behaviour signals</t>
+        </is>
+      </c>
+      <c r="F199" s="7" t="inlineStr">
+        <is>
+          <t>From $49/user/mo</t>
+        </is>
+      </c>
+      <c r="G199" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H199" s="7" t="inlineStr">
+        <is>
+          <t>Automatic CRM hygiene; emotion/engagement signals</t>
+        </is>
+      </c>
+      <c r="I199" s="7" t="inlineStr">
+        <is>
+          <t>Per-seat cost; niche</t>
+        </is>
+      </c>
+      <c r="J199" s="7" t="inlineStr">
+        <is>
+          <t>AEs hating CRM data entry</t>
+        </is>
+      </c>
+      <c r="K199" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L199" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="M199" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N199" s="5" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="O199" s="5" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="200" ht="58" customHeight="1">
+      <c r="A200" s="9">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B200" s="10" t="inlineStr">
+        <is>
+          <t>Twenty</t>
+        </is>
+      </c>
+      <c r="C200" s="11" t="inlineStr">
+        <is>
+          <t>Open source (GitHub)</t>
+        </is>
+      </c>
+      <c r="D200" s="12" t="inlineStr">
+        <is>
+          <t>github.com/twentyhq/twenty</t>
+        </is>
+      </c>
+      <c r="E200" s="11" t="inlineStr">
+        <is>
+          <t>Modern open-source CRM (the OSS Salesforce alternative)</t>
+        </is>
+      </c>
+      <c r="F200" s="11" t="inlineStr">
+        <is>
+          <t>Free self-host; cloud from $9/user/mo</t>
+        </is>
+      </c>
+      <c r="G200" s="11" t="inlineStr">
+        <is>
+          <t>Partial — API/webhooks; community MCP</t>
+        </is>
+      </c>
+      <c r="H200" s="11" t="inlineStr">
+        <is>
+          <t>Beautiful modern OSS CRM; data ownership</t>
+        </is>
+      </c>
+      <c r="I200" s="11" t="inlineStr">
+        <is>
+          <t>Younger ecosystem; fewer native integrations</t>
+        </is>
+      </c>
+      <c r="J200" s="11" t="inlineStr">
+        <is>
+          <t>Startups wanting an ownable CRM</t>
+        </is>
+      </c>
+      <c r="K200" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L200" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="M200" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="N200" s="9" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="O200" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="201" ht="58" customHeight="1">
+      <c r="A201" s="9">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B201" s="10" t="inlineStr">
+        <is>
+          <t>EspoCRM</t>
+        </is>
+      </c>
+      <c r="C201" s="11" t="inlineStr">
+        <is>
+          <t>Open source (GitHub)</t>
+        </is>
+      </c>
+      <c r="D201" s="12" t="inlineStr">
+        <is>
+          <t>github.com/espocrm/espocrm</t>
+        </is>
+      </c>
+      <c r="E201" s="11" t="inlineStr">
+        <is>
+          <t>Mature open-source CRM with workflows and email</t>
+        </is>
+      </c>
+      <c r="F201" s="11" t="inlineStr">
+        <is>
+          <t>Free self-host; cloud from $15/mo</t>
+        </is>
+      </c>
+      <c r="G201" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H201" s="11" t="inlineStr">
+        <is>
+          <t>Proven, full-featured, cheap</t>
+        </is>
+      </c>
+      <c r="I201" s="11" t="inlineStr">
+        <is>
+          <t>Dated UI; AI minimal</t>
+        </is>
+      </c>
+      <c r="J201" s="11" t="inlineStr">
+        <is>
+          <t>Cost-sensitive sales teams</t>
+        </is>
+      </c>
+      <c r="K201" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L201" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="M201" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N201" s="9" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="O201" s="9" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="202" ht="58" customHeight="1">
+      <c r="A202" s="9">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B202" s="10" t="inlineStr">
+        <is>
+          <t>Frappe CRM</t>
+        </is>
+      </c>
+      <c r="C202" s="11" t="inlineStr">
+        <is>
+          <t>Open source (GitHub)</t>
+        </is>
+      </c>
+      <c r="D202" s="12" t="inlineStr">
+        <is>
+          <t>github.com/frappe/crm</t>
+        </is>
+      </c>
+      <c r="E202" s="11" t="inlineStr">
+        <is>
+          <t>Clean open-source CRM from the ERPNext ecosystem</t>
+        </is>
+      </c>
+      <c r="F202" s="11" t="inlineStr">
+        <is>
+          <t>Free self-host; cloud plans</t>
+        </is>
+      </c>
+      <c r="G202" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H202" s="11" t="inlineStr">
+        <is>
+          <t>Modern UX; ERPNext integration</t>
+        </is>
+      </c>
+      <c r="I202" s="11" t="inlineStr">
+        <is>
+          <t>Smaller community</t>
+        </is>
+      </c>
+      <c r="J202" s="11" t="inlineStr">
+        <is>
+          <t>Companies already on Frappe/ERPNext</t>
+        </is>
+      </c>
+      <c r="K202" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L202" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="M202" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="N202" s="9" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="O202" s="9" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="196" ht="58" customHeight="1">
-      <c r="A196" s="9">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B196" s="10" t="inlineStr">
-        <is>
-          <t>Twenty</t>
-        </is>
-      </c>
-      <c r="C196" s="11" t="inlineStr">
-        <is>
-          <t>Open source (GitHub)</t>
-        </is>
-      </c>
-      <c r="D196" s="12" t="inlineStr">
-        <is>
-          <t>github.com/twentyhq/twenty</t>
-        </is>
-      </c>
-      <c r="E196" s="11" t="inlineStr">
-        <is>
-          <t>Modern open-source CRM (the OSS Salesforce alternative)</t>
-        </is>
-      </c>
-      <c r="F196" s="11" t="inlineStr">
-        <is>
-          <t>Free self-host; cloud from $9/user/mo</t>
-        </is>
-      </c>
-      <c r="G196" s="11" t="inlineStr">
-        <is>
-          <t>Partial — API/webhooks; community MCP</t>
-        </is>
-      </c>
-      <c r="H196" s="11" t="inlineStr">
-        <is>
-          <t>Beautiful modern OSS CRM; data ownership</t>
-        </is>
-      </c>
-      <c r="I196" s="11" t="inlineStr">
-        <is>
-          <t>Younger ecosystem; fewer native integrations</t>
-        </is>
-      </c>
-      <c r="J196" s="11" t="inlineStr">
-        <is>
-          <t>Startups wanting an ownable CRM</t>
-        </is>
-      </c>
-      <c r="K196" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="L196" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="M196" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="N196" s="9" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="O196" s="9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="197" ht="58" customHeight="1">
-      <c r="A197" s="9">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B197" s="10" t="inlineStr">
-        <is>
-          <t>EspoCRM</t>
-        </is>
-      </c>
-      <c r="C197" s="11" t="inlineStr">
-        <is>
-          <t>Open source (GitHub)</t>
-        </is>
-      </c>
-      <c r="D197" s="12" t="inlineStr">
-        <is>
-          <t>github.com/espocrm/espocrm</t>
-        </is>
-      </c>
-      <c r="E197" s="11" t="inlineStr">
-        <is>
-          <t>Mature open-source CRM with workflows and email</t>
-        </is>
-      </c>
-      <c r="F197" s="11" t="inlineStr">
-        <is>
-          <t>Free self-host; cloud from $15/mo</t>
-        </is>
-      </c>
-      <c r="G197" s="11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H197" s="11" t="inlineStr">
-        <is>
-          <t>Proven, full-featured, cheap</t>
-        </is>
-      </c>
-      <c r="I197" s="11" t="inlineStr">
-        <is>
-          <t>Dated UI; AI minimal</t>
-        </is>
-      </c>
-      <c r="J197" s="11" t="inlineStr">
-        <is>
-          <t>Cost-sensitive sales teams</t>
-        </is>
-      </c>
-      <c r="K197" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="L197" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="M197" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N197" s="9" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="O197" s="9" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="198" ht="58" customHeight="1">
-      <c r="A198" s="9">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B198" s="10" t="inlineStr">
-        <is>
-          <t>Frappe CRM</t>
-        </is>
-      </c>
-      <c r="C198" s="11" t="inlineStr">
-        <is>
-          <t>Open source (GitHub)</t>
-        </is>
-      </c>
-      <c r="D198" s="12" t="inlineStr">
-        <is>
-          <t>github.com/frappe/crm</t>
-        </is>
-      </c>
-      <c r="E198" s="11" t="inlineStr">
-        <is>
-          <t>Clean open-source CRM from the ERPNext ecosystem</t>
-        </is>
-      </c>
-      <c r="F198" s="11" t="inlineStr">
-        <is>
-          <t>Free self-host; cloud plans</t>
-        </is>
-      </c>
-      <c r="G198" s="11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H198" s="11" t="inlineStr">
-        <is>
-          <t>Modern UX; ERPNext integration</t>
-        </is>
-      </c>
-      <c r="I198" s="11" t="inlineStr">
-        <is>
-          <t>Smaller community</t>
-        </is>
-      </c>
-      <c r="J198" s="11" t="inlineStr">
-        <is>
-          <t>Companies already on Frappe/ERPNext</t>
-        </is>
-      </c>
-      <c r="K198" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="L198" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="M198" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="N198" s="9" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="O198" s="9" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="199" ht="22" customHeight="1">
-      <c r="A199" s="4" t="inlineStr">
-        <is>
-          <t>AI Marketing &amp; SEO</t>
-        </is>
-      </c>
-    </row>
-    <row r="200" ht="58" customHeight="1">
-      <c r="A200" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=semrush.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B200" s="6" t="inlineStr">
-        <is>
-          <t>Semrush</t>
-        </is>
-      </c>
-      <c r="C200" s="7" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="D200" s="8" t="inlineStr">
-        <is>
-          <t>semrush.com</t>
-        </is>
-      </c>
-      <c r="E200" s="7" t="inlineStr">
-        <is>
-          <t>All-in-one SEO/SEM platform with AI features and ContentShake</t>
-        </is>
-      </c>
-      <c r="F200" s="7" t="inlineStr">
-        <is>
-          <t>From $139.95/mo</t>
-        </is>
-      </c>
-      <c r="G200" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H200" s="7" t="inlineStr">
-        <is>
-          <t>Deepest SEO dataset; AI content tools</t>
-        </is>
-      </c>
-      <c r="I200" s="7" t="inlineStr">
-        <is>
-          <t>Expensive; overwhelming</t>
-        </is>
-      </c>
-      <c r="J200" s="7" t="inlineStr">
-        <is>
-          <t>SEO professionals</t>
-        </is>
-      </c>
-      <c r="K200" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="L200" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="M200" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="N200" s="5" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="O200" s="5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="201" ht="58" customHeight="1">
-      <c r="A201" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=ahrefs.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B201" s="6" t="inlineStr">
-        <is>
-          <t>Ahrefs</t>
-        </is>
-      </c>
-      <c r="C201" s="7" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="D201" s="8" t="inlineStr">
-        <is>
-          <t>ahrefs.com</t>
-        </is>
-      </c>
-      <c r="E201" s="7" t="inlineStr">
-        <is>
-          <t>Backlink/keyword research leader with AI content helper</t>
-        </is>
-      </c>
-      <c r="F201" s="7" t="inlineStr">
-        <is>
-          <t>From $129/mo</t>
-        </is>
-      </c>
-      <c r="G201" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H201" s="7" t="inlineStr">
-        <is>
-          <t>Best link data; clean UX</t>
-        </is>
-      </c>
-      <c r="I201" s="7" t="inlineStr">
-        <is>
-          <t>No free tier; AI is light</t>
-        </is>
-      </c>
-      <c r="J201" s="7" t="inlineStr">
-        <is>
-          <t>Link-building and SEO research</t>
-        </is>
-      </c>
-      <c r="K201" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="L201" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="M201" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="N201" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="O201" s="5" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="202" ht="58" customHeight="1">
-      <c r="A202" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=surferseo.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B202" s="6" t="inlineStr">
-        <is>
-          <t>Surfer</t>
-        </is>
-      </c>
-      <c r="C202" s="7" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="D202" s="8" t="inlineStr">
-        <is>
-          <t>surferseo.com</t>
-        </is>
-      </c>
-      <c r="E202" s="7" t="inlineStr">
-        <is>
-          <t>On-page SEO content optimisation with AI writing</t>
-        </is>
-      </c>
-      <c r="F202" s="7" t="inlineStr">
-        <is>
-          <t>From $89/mo</t>
-        </is>
-      </c>
-      <c r="G202" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H202" s="7" t="inlineStr">
-        <is>
-          <t>Clear data-driven content scores</t>
-        </is>
-      </c>
-      <c r="I202" s="7" t="inlineStr">
-        <is>
-          <t>Per-article economics; SERP-chasing risk</t>
-        </is>
-      </c>
-      <c r="J202" s="7" t="inlineStr">
-        <is>
-          <t>Content teams optimising for Google</t>
-        </is>
-      </c>
-      <c r="K202" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="L202" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="M202" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="N202" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="O202" s="5" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="203" ht="58" customHeight="1">
-      <c r="A203" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=adcreative.ai&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B203" s="6" t="inlineStr">
-        <is>
-          <t>AdCreative.ai</t>
-        </is>
-      </c>
-      <c r="C203" s="7" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="D203" s="8" t="inlineStr">
-        <is>
-          <t>adcreative.ai</t>
-        </is>
-      </c>
-      <c r="E203" s="7" t="inlineStr">
-        <is>
-          <t>AI ad creative and copy generation with performance scoring</t>
-        </is>
-      </c>
-      <c r="F203" s="7" t="inlineStr">
-        <is>
-          <t>From $25/mo</t>
-        </is>
-      </c>
-      <c r="G203" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H203" s="7" t="inlineStr">
-        <is>
-          <t>Volume ad-variant generation; scoring</t>
-        </is>
-      </c>
-      <c r="I203" s="7" t="inlineStr">
-        <is>
-          <t>Template look; aggressive billing reputation — check terms</t>
-        </is>
-      </c>
-      <c r="J203" s="7" t="inlineStr">
-        <is>
-          <t>Performance marketers</t>
-        </is>
-      </c>
-      <c r="K203" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="L203" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="M203" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N203" s="5" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="O203" s="5" t="n">
-        <v>9</v>
+    <row r="203" ht="22" customHeight="1">
+      <c r="A203" s="4" t="inlineStr">
+        <is>
+          <t>AI Sales Outreach &amp; Prospecting</t>
+        </is>
       </c>
     </row>
     <row r="204" ht="58" customHeight="1">
       <c r="A204" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=hootsuite.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=zoominfo.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B204" s="6" t="inlineStr">
         <is>
-          <t>Hootsuite</t>
+          <t>ZoomInfo Copilot</t>
         </is>
       </c>
       <c r="C204" s="7" t="inlineStr">
@@ -13122,17 +13122,17 @@
       </c>
       <c r="D204" s="8" t="inlineStr">
         <is>
-          <t>hootsuite.com</t>
+          <t>zoominfo.com</t>
         </is>
       </c>
       <c r="E204" s="7" t="inlineStr">
         <is>
-          <t>Social media management with OwlyWriter AI</t>
+          <t>B2B contact/company database with intent data and an AI copilot</t>
         </is>
       </c>
       <c r="F204" s="7" t="inlineStr">
         <is>
-          <t>From $99/mo</t>
+          <t>From ~$15k/yr (contract)</t>
         </is>
       </c>
       <c r="G204" s="7" t="inlineStr">
@@ -13142,43 +13142,43 @@
       </c>
       <c r="H204" s="7" t="inlineStr">
         <is>
-          <t>Mature scheduling/listening suite</t>
+          <t>Deepest B2B data + buying-intent signals</t>
         </is>
       </c>
       <c r="I204" s="7" t="inlineStr">
         <is>
-          <t>Expensive; AI basic</t>
+          <t>Expensive annual contracts</t>
         </is>
       </c>
       <c r="J204" s="7" t="inlineStr">
         <is>
-          <t>Social teams managing many accounts</t>
+          <t>Enterprise outbound teams</t>
         </is>
       </c>
       <c r="K204" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L204" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M204" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="N204" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="O204" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="M204" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="N204" s="5" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="O204" s="5" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="205" ht="58" customHeight="1">
       <c r="A205" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=buffer.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=lusha.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B205" s="6" t="inlineStr">
         <is>
-          <t>Buffer</t>
+          <t>Lusha</t>
         </is>
       </c>
       <c r="C205" s="7" t="inlineStr">
@@ -13188,17 +13188,17 @@
       </c>
       <c r="D205" s="8" t="inlineStr">
         <is>
-          <t>buffer.com</t>
+          <t>lusha.com</t>
         </is>
       </c>
       <c r="E205" s="7" t="inlineStr">
         <is>
-          <t>Simple social scheduling with AI assistant</t>
+          <t>B2B contact data via web app and Chrome extension</t>
         </is>
       </c>
       <c r="F205" s="7" t="inlineStr">
         <is>
-          <t>Free; $6/channel/mo</t>
+          <t>Free; from $36/user/mo</t>
         </is>
       </c>
       <c r="G205" s="7" t="inlineStr">
@@ -13208,43 +13208,43 @@
       </c>
       <c r="H205" s="7" t="inlineStr">
         <is>
-          <t>Affordable; clean; good AI repurposing</t>
+          <t>Easy to use; compliance-focused data</t>
         </is>
       </c>
       <c r="I205" s="7" t="inlineStr">
         <is>
-          <t>Lighter analytics</t>
+          <t>Smaller database than ZoomInfo</t>
         </is>
       </c>
       <c r="J205" s="7" t="inlineStr">
         <is>
-          <t>Creators and small brands</t>
+          <t>SDRs needing quick contact data</t>
         </is>
       </c>
       <c r="K205" s="5" t="n">
         <v>5</v>
       </c>
       <c r="L205" s="5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M205" s="5" t="n">
         <v>6</v>
       </c>
       <c r="N205" s="5" t="n">
-        <v>6.3</v>
+        <v>5.7</v>
       </c>
       <c r="O205" s="5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="206" ht="58" customHeight="1">
       <c r="A206" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=mailchimp.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=seamless.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B206" s="6" t="inlineStr">
         <is>
-          <t>Mailchimp</t>
+          <t>Seamless.AI</t>
         </is>
       </c>
       <c r="C206" s="7" t="inlineStr">
@@ -13254,17 +13254,17 @@
       </c>
       <c r="D206" s="8" t="inlineStr">
         <is>
-          <t>mailchimp.com</t>
+          <t>seamless.ai</t>
         </is>
       </c>
       <c r="E206" s="7" t="inlineStr">
         <is>
-          <t>Email marketing with AI content and journeys</t>
+          <t>Real-time AI search engine for B2B contact information</t>
         </is>
       </c>
       <c r="F206" s="7" t="inlineStr">
         <is>
-          <t>Free; from $13/mo</t>
+          <t>Free credits; from ~$147/mo</t>
         </is>
       </c>
       <c r="G206" s="7" t="inlineStr">
@@ -13274,334 +13274,393 @@
       </c>
       <c r="H206" s="7" t="inlineStr">
         <is>
-          <t>Familiar; AI campaign generation</t>
+          <t>Real-time verification; high volumes</t>
         </is>
       </c>
       <c r="I206" s="7" t="inlineStr">
         <is>
-          <t>Pricing grows with list; CRM-lite</t>
+          <t>Data-accuracy complaints; pushy sales motion</t>
         </is>
       </c>
       <c r="J206" s="7" t="inlineStr">
         <is>
-          <t>SMB email marketing</t>
+          <t>High-volume prospectors</t>
         </is>
       </c>
       <c r="K206" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L206" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M206" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N206" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="O206" s="5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="207" ht="58" customHeight="1">
+      <c r="A207" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=instantly.ai&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B207" s="6" t="inlineStr">
+        <is>
+          <t>Instantly</t>
+        </is>
+      </c>
+      <c r="C207" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D207" s="8" t="inlineStr">
+        <is>
+          <t>instantly.ai</t>
+        </is>
+      </c>
+      <c r="E207" s="7" t="inlineStr">
+        <is>
+          <t>Cold email at scale: warmup, inbox rotation, deliverability, AI writing</t>
+        </is>
+      </c>
+      <c r="F207" s="7" t="inlineStr">
+        <is>
+          <t>From $37/mo</t>
+        </is>
+      </c>
+      <c r="G207" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H207" s="7" t="inlineStr">
+        <is>
+          <t>Best-known deliverability stack; unlimited sending accounts</t>
+        </is>
+      </c>
+      <c r="I207" s="7" t="inlineStr">
+        <is>
+          <t>Cold-email compliance is on you</t>
+        </is>
+      </c>
+      <c r="J207" s="7" t="inlineStr">
+        <is>
+          <t>Agencies and outbound startups</t>
+        </is>
+      </c>
+      <c r="K207" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L207" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="M207" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N207" s="5" t="n">
         <v>6.3</v>
       </c>
-      <c r="O206" s="5" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="207" ht="58" customHeight="1">
-      <c r="A207" s="9">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B207" s="10" t="inlineStr">
-        <is>
-          <t>Mautic</t>
-        </is>
-      </c>
-      <c r="C207" s="11" t="inlineStr">
-        <is>
-          <t>Open source (GitHub)</t>
-        </is>
-      </c>
-      <c r="D207" s="12" t="inlineStr">
-        <is>
-          <t>github.com/mautic/mautic</t>
-        </is>
-      </c>
-      <c r="E207" s="11" t="inlineStr">
-        <is>
-          <t>Open-source marketing automation (email, journeys, segmentation)</t>
-        </is>
-      </c>
-      <c r="F207" s="11" t="inlineStr">
-        <is>
-          <t>Free (self-host)</t>
-        </is>
-      </c>
-      <c r="G207" s="11" t="inlineStr">
+      <c r="O207" s="5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="208" ht="58" customHeight="1">
+      <c r="A208" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=smartlead.ai&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B208" s="6" t="inlineStr">
+        <is>
+          <t>Smartlead</t>
+        </is>
+      </c>
+      <c r="C208" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D208" s="8" t="inlineStr">
+        <is>
+          <t>smartlead.ai</t>
+        </is>
+      </c>
+      <c r="E208" s="7" t="inlineStr">
+        <is>
+          <t>Cold email infrastructure with unlimited mailboxes and AI warmup</t>
+        </is>
+      </c>
+      <c r="F208" s="7" t="inlineStr">
+        <is>
+          <t>From $39/mo</t>
+        </is>
+      </c>
+      <c r="G208" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H207" s="11" t="inlineStr">
-        <is>
-          <t>Full marketing automation without per-contact fees</t>
-        </is>
-      </c>
-      <c r="I207" s="11" t="inlineStr">
-        <is>
-          <t>Self-host complexity; plugins needed</t>
-        </is>
-      </c>
-      <c r="J207" s="11" t="inlineStr">
-        <is>
-          <t>Companies escaping HubSpot/Marketo pricing</t>
-        </is>
-      </c>
-      <c r="K207" s="9" t="n">
+      <c r="H208" s="7" t="inlineStr">
+        <is>
+          <t>Unlimited mailboxes; API-first</t>
+        </is>
+      </c>
+      <c r="I208" s="7" t="inlineStr">
+        <is>
+          <t>UI rough edges</t>
+        </is>
+      </c>
+      <c r="J208" s="7" t="inlineStr">
+        <is>
+          <t>Outbound agencies</t>
+        </is>
+      </c>
+      <c r="K208" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="L207" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="M207" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="N207" s="9" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="O207" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="208" ht="58" customHeight="1">
-      <c r="A208" s="9">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B208" s="10" t="inlineStr">
-        <is>
-          <t>Postiz</t>
-        </is>
-      </c>
-      <c r="C208" s="11" t="inlineStr">
-        <is>
-          <t>Open source (GitHub)</t>
-        </is>
-      </c>
-      <c r="D208" s="12" t="inlineStr">
-        <is>
-          <t>github.com/gitroomhq/postiz-app</t>
-        </is>
-      </c>
-      <c r="E208" s="11" t="inlineStr">
-        <is>
-          <t>Open-source AI social media scheduling (Buffer/Hootsuite alternative)</t>
-        </is>
-      </c>
-      <c r="F208" s="11" t="inlineStr">
-        <is>
-          <t>Free self-host; cloud from $29/mo</t>
-        </is>
-      </c>
-      <c r="G208" s="11" t="inlineStr">
-        <is>
-          <t>Partial — BYO AI keys</t>
-        </is>
-      </c>
-      <c r="H208" s="11" t="inlineStr">
-        <is>
-          <t>OSS scheduling for 15+ platforms with AI</t>
-        </is>
-      </c>
-      <c r="I208" s="11" t="inlineStr">
-        <is>
-          <t>Young project</t>
-        </is>
-      </c>
-      <c r="J208" s="11" t="inlineStr">
-        <is>
-          <t>Self-hosted social scheduling</t>
-        </is>
-      </c>
-      <c r="K208" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="L208" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="M208" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N208" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="O208" s="9" t="n">
-        <v>2</v>
+      <c r="L208" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="M208" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N208" s="5" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="O208" s="5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="209" ht="58" customHeight="1">
-      <c r="A209" s="9">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B209" s="10" t="inlineStr">
-        <is>
-          <t>Matomo</t>
-        </is>
-      </c>
-      <c r="C209" s="11" t="inlineStr">
-        <is>
-          <t>Open source (GitHub)</t>
-        </is>
-      </c>
-      <c r="D209" s="12" t="inlineStr">
-        <is>
-          <t>github.com/matomo-org/matomo</t>
-        </is>
-      </c>
-      <c r="E209" s="11" t="inlineStr">
-        <is>
-          <t>Open-source web analytics (Google Analytics alternative)</t>
-        </is>
-      </c>
-      <c r="F209" s="11" t="inlineStr">
-        <is>
-          <t>Free self-host; cloud from $23/mo</t>
-        </is>
-      </c>
-      <c r="G209" s="11" t="inlineStr">
+      <c r="A209" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=lemlist.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B209" s="6" t="inlineStr">
+        <is>
+          <t>lemlist</t>
+        </is>
+      </c>
+      <c r="C209" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D209" s="8" t="inlineStr">
+        <is>
+          <t>lemlist.com</t>
+        </is>
+      </c>
+      <c r="E209" s="7" t="inlineStr">
+        <is>
+          <t>Multichannel outreach (email/LinkedIn/calls) with AI personalisation</t>
+        </is>
+      </c>
+      <c r="F209" s="7" t="inlineStr">
+        <is>
+          <t>From $39/user/mo</t>
+        </is>
+      </c>
+      <c r="G209" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H209" s="11" t="inlineStr">
-        <is>
-          <t>Privacy-compliant analytics you own</t>
-        </is>
-      </c>
-      <c r="I209" s="11" t="inlineStr">
-        <is>
-          <t>No AI insights layer yet</t>
-        </is>
-      </c>
-      <c r="J209" s="11" t="inlineStr">
-        <is>
-          <t>Privacy-first site analytics</t>
-        </is>
-      </c>
-      <c r="K209" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="L209" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="M209" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="N209" s="9" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="O209" s="9" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="210" ht="22" customHeight="1">
-      <c r="A210" s="4" t="inlineStr">
-        <is>
-          <t>AI Research Tools</t>
-        </is>
+      <c r="H209" s="7" t="inlineStr">
+        <is>
+          <t>Strong personalisation (images, dynamic content)</t>
+        </is>
+      </c>
+      <c r="I209" s="7" t="inlineStr">
+        <is>
+          <t>Per-seat costs add up</t>
+        </is>
+      </c>
+      <c r="J209" s="7" t="inlineStr">
+        <is>
+          <t>SDRs doing personalised sequences</t>
+        </is>
+      </c>
+      <c r="K209" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L209" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M209" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N209" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="O209" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="210" ht="58" customHeight="1">
+      <c r="A210" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=reply.io&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B210" s="6" t="inlineStr">
+        <is>
+          <t>Reply.io</t>
+        </is>
+      </c>
+      <c r="C210" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D210" s="8" t="inlineStr">
+        <is>
+          <t>reply.io</t>
+        </is>
+      </c>
+      <c r="E210" s="7" t="inlineStr">
+        <is>
+          <t>AI SDR agents plus multichannel sales sequences</t>
+        </is>
+      </c>
+      <c r="F210" s="7" t="inlineStr">
+        <is>
+          <t>From $59/user/mo; AI SDR from ~$259/mo</t>
+        </is>
+      </c>
+      <c r="G210" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H210" s="7" t="inlineStr">
+        <is>
+          <t>Mature sequencer with AI-agent option</t>
+        </is>
+      </c>
+      <c r="I210" s="7" t="inlineStr">
+        <is>
+          <t>AI-agent quality varies</t>
+        </is>
+      </c>
+      <c r="J210" s="7" t="inlineStr">
+        <is>
+          <t>Lean teams automating outreach</t>
+        </is>
+      </c>
+      <c r="K210" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L210" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M210" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N210" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="O210" s="5" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="211" ht="58" customHeight="1">
       <c r="A211" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=elicit.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=qualified.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B211" s="6" t="inlineStr">
         <is>
-          <t>Elicit</t>
+          <t>Qualified</t>
         </is>
       </c>
       <c r="C211" s="7" t="inlineStr">
         <is>
-          <t>Freemium</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="D211" s="8" t="inlineStr">
         <is>
-          <t>elicit.com</t>
+          <t>qualified.com</t>
         </is>
       </c>
       <c r="E211" s="7" t="inlineStr">
         <is>
-          <t>AI research assistant that searches and summarises academic papers</t>
+          <t>AI SDR 'Piper' converts website visitors into pipeline (Salesforce-native)</t>
         </is>
       </c>
       <c r="F211" s="7" t="inlineStr">
         <is>
-          <t>Free; Plus $12/mo</t>
+          <t>From ~$3,500/mo</t>
         </is>
       </c>
       <c r="G211" s="7" t="inlineStr">
         <is>
-          <t>No — (Anthropic models used under the hood historically)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H211" s="7" t="inlineStr">
         <is>
-          <t>Systematic-review-grade extraction tables</t>
+          <t>Best-in-class inbound conversion for Salesforce shops</t>
         </is>
       </c>
       <c r="I211" s="7" t="inlineStr">
         <is>
-          <t>Academic papers only</t>
+          <t>Enterprise pricing; Salesforce required</t>
         </is>
       </c>
       <c r="J211" s="7" t="inlineStr">
         <is>
-          <t>Researchers and grad students</t>
+          <t>Enterprise demand-gen teams</t>
         </is>
       </c>
       <c r="K211" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L211" s="5" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M211" s="5" t="n">
         <v>8</v>
       </c>
       <c r="N211" s="5" t="n">
-        <v>6.7</v>
+        <v>5.7</v>
       </c>
       <c r="O211" s="5" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="212" ht="58" customHeight="1">
       <c r="A212" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=consensus.app&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=11x.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B212" s="6" t="inlineStr">
         <is>
-          <t>Consensus</t>
+          <t>11x</t>
         </is>
       </c>
       <c r="C212" s="7" t="inlineStr">
         <is>
-          <t>Freemium</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="D212" s="8" t="inlineStr">
         <is>
-          <t>consensus.app</t>
+          <t>11x.ai</t>
         </is>
       </c>
       <c r="E212" s="7" t="inlineStr">
         <is>
-          <t>Search engine answering questions from peer-reviewed evidence</t>
+          <t>Autonomous 'digital worker' AI SDRs (Alice) running outbound end-to-end</t>
         </is>
       </c>
       <c r="F212" s="7" t="inlineStr">
         <is>
-          <t>Free; Premium $11.99/mo</t>
+          <t>Custom (thousands/mo)</t>
         </is>
       </c>
       <c r="G212" s="7" t="inlineStr">
@@ -13611,63 +13670,63 @@
       </c>
       <c r="H212" s="7" t="inlineStr">
         <is>
-          <t>Evidence meters; citation-grounded answers</t>
+          <t>Fully autonomous outbound experiments</t>
         </is>
       </c>
       <c r="I212" s="7" t="inlineStr">
         <is>
-          <t>Narrower than general search</t>
+          <t>Mixed quality reports; hype-heavy category</t>
         </is>
       </c>
       <c r="J212" s="7" t="inlineStr">
         <is>
-          <t>Evidence-based professionals</t>
+          <t>Teams experimenting with AI SDRs</t>
         </is>
       </c>
       <c r="K212" s="5" t="n">
         <v>4</v>
       </c>
       <c r="L212" s="5" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M212" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N212" s="5" t="n">
-        <v>6</v>
+        <v>4.3</v>
       </c>
       <c r="O212" s="5" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="213" ht="58" customHeight="1">
       <c r="A213" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=scispace.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=artisan.co&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B213" s="6" t="inlineStr">
         <is>
-          <t>SciSpace</t>
+          <t>Artisan</t>
         </is>
       </c>
       <c r="C213" s="7" t="inlineStr">
         <is>
-          <t>Freemium</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="D213" s="8" t="inlineStr">
         <is>
-          <t>scispace.com</t>
+          <t>artisan.co</t>
         </is>
       </c>
       <c r="E213" s="7" t="inlineStr">
         <is>
-          <t>Read, annotate and chat with research PDFs; literature review AI</t>
+          <t>AI BDR 'Ava': finds leads, researches, writes and sends outbound</t>
         </is>
       </c>
       <c r="F213" s="7" t="inlineStr">
         <is>
-          <t>Free; from $12/mo</t>
+          <t>Custom (from ~$2k/mo)</t>
         </is>
       </c>
       <c r="G213" s="7" t="inlineStr">
@@ -13677,187 +13736,1390 @@
       </c>
       <c r="H213" s="7" t="inlineStr">
         <is>
-          <t>Great PDF explanation UX</t>
+          <t>Consolidates data + email infra + AI in one</t>
         </is>
       </c>
       <c r="I213" s="7" t="inlineStr">
         <is>
-          <t>Aggressive upsells</t>
+          <t>Young product; needs supervision</t>
         </is>
       </c>
       <c r="J213" s="7" t="inlineStr">
         <is>
-          <t>Students decoding dense papers</t>
+          <t>Startups without SDR headcount</t>
         </is>
       </c>
       <c r="K213" s="5" t="n">
         <v>4</v>
       </c>
       <c r="L213" s="5" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M213" s="5" t="n">
         <v>6</v>
       </c>
       <c r="N213" s="5" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="O213" s="5" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="214" ht="58" customHeight="1">
+      <c r="A214" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=nooks.ai&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B214" s="6" t="inlineStr">
+        <is>
+          <t>Nooks</t>
+        </is>
+      </c>
+      <c r="C214" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D214" s="8" t="inlineStr">
+        <is>
+          <t>nooks.ai</t>
+        </is>
+      </c>
+      <c r="E214" s="7" t="inlineStr">
+        <is>
+          <t>AI parallel dialer, virtual salesfloor and call coaching</t>
+        </is>
+      </c>
+      <c r="F214" s="7" t="inlineStr">
+        <is>
+          <t>Custom (~$200/user/mo)</t>
+        </is>
+      </c>
+      <c r="G214" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H214" s="7" t="inlineStr">
+        <is>
+          <t>3-5x connect rates for calling teams</t>
+        </is>
+      </c>
+      <c r="I214" s="7" t="inlineStr">
+        <is>
+          <t>Dialer-centric; custom pricing</t>
+        </is>
+      </c>
+      <c r="J214" s="7" t="inlineStr">
+        <is>
+          <t>Cold-calling SDR teams</t>
+        </is>
+      </c>
+      <c r="K214" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L214" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M214" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N214" s="5" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="O214" s="5" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="215" ht="58" customHeight="1">
+      <c r="A215" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=warmly.ai&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B215" s="6" t="inlineStr">
+        <is>
+          <t>Warmly</t>
+        </is>
+      </c>
+      <c r="C215" s="7" t="inlineStr">
+        <is>
+          <t>Freemium</t>
+        </is>
+      </c>
+      <c r="D215" s="8" t="inlineStr">
+        <is>
+          <t>warmly.ai</t>
+        </is>
+      </c>
+      <c r="E215" s="7" t="inlineStr">
+        <is>
+          <t>De-anonymises website visitors and orchestrates AI outreach to them</t>
+        </is>
+      </c>
+      <c r="F215" s="7" t="inlineStr">
+        <is>
+          <t>Free; from ~$700/mo</t>
+        </is>
+      </c>
+      <c r="G215" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H215" s="7" t="inlineStr">
+        <is>
+          <t>Good intent signals for the price</t>
+        </is>
+      </c>
+      <c r="I215" s="7" t="inlineStr">
+        <is>
+          <t>Pricing jumps sharply after free tier</t>
+        </is>
+      </c>
+      <c r="J215" s="7" t="inlineStr">
+        <is>
+          <t>SMB pipeline teams</t>
+        </is>
+      </c>
+      <c r="K215" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L215" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="M215" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N215" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="O215" s="5" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="216" ht="58" customHeight="1">
+      <c r="A216" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=crystalknows.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B216" s="6" t="inlineStr">
+        <is>
+          <t>Crystal</t>
+        </is>
+      </c>
+      <c r="C216" s="7" t="inlineStr">
+        <is>
+          <t>Freemium</t>
+        </is>
+      </c>
+      <c r="D216" s="8" t="inlineStr">
+        <is>
+          <t>crystalknows.com</t>
+        </is>
+      </c>
+      <c r="E216" s="7" t="inlineStr">
+        <is>
+          <t>DISC personality profiles for prospects to tailor messaging</t>
+        </is>
+      </c>
+      <c r="F216" s="7" t="inlineStr">
+        <is>
+          <t>Free; from $49/mo</t>
+        </is>
+      </c>
+      <c r="G216" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H216" s="7" t="inlineStr">
+        <is>
+          <t>Unique personality-based angle</t>
+        </is>
+      </c>
+      <c r="I216" s="7" t="inlineStr">
+        <is>
+          <t>Profile accuracy varies</t>
+        </is>
+      </c>
+      <c r="J216" s="7" t="inlineStr">
+        <is>
+          <t>Relationship-driven sellers</t>
+        </is>
+      </c>
+      <c r="K216" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L216" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="M216" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N216" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="O216" s="5" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="217" ht="58" customHeight="1">
+      <c r="A217" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=regie.ai&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B217" s="6" t="inlineStr">
+        <is>
+          <t>Regie.ai</t>
+        </is>
+      </c>
+      <c r="C217" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D217" s="8" t="inlineStr">
+        <is>
+          <t>regie.ai</t>
+        </is>
+      </c>
+      <c r="E217" s="7" t="inlineStr">
+        <is>
+          <t>Generative AI platform for sales prospecting content and sequencing</t>
+        </is>
+      </c>
+      <c r="F217" s="7" t="inlineStr">
+        <is>
+          <t>Custom pricing</t>
+        </is>
+      </c>
+      <c r="G217" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H217" s="7" t="inlineStr">
+        <is>
+          <t>Brand-controlled AI sales content at scale</t>
+        </is>
+      </c>
+      <c r="I217" s="7" t="inlineStr">
+        <is>
+          <t>Opaque pricing</t>
+        </is>
+      </c>
+      <c r="J217" s="7" t="inlineStr">
+        <is>
+          <t>Enterprise SDR organisations</t>
+        </is>
+      </c>
+      <c r="K217" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L217" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M217" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N217" s="5" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="O217" s="5" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="218" ht="58" customHeight="1">
+      <c r="A218" s="9">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B218" s="10" t="inlineStr">
+        <is>
+          <t>Listmonk</t>
+        </is>
+      </c>
+      <c r="C218" s="11" t="inlineStr">
+        <is>
+          <t>Open source (GitHub)</t>
+        </is>
+      </c>
+      <c r="D218" s="12" t="inlineStr">
+        <is>
+          <t>github.com/knadh/listmonk</t>
+        </is>
+      </c>
+      <c r="E218" s="11" t="inlineStr">
+        <is>
+          <t>Self-hosted high-performance email campaign and newsletter manager</t>
+        </is>
+      </c>
+      <c r="F218" s="11" t="inlineStr">
+        <is>
+          <t>Free (self-host)</t>
+        </is>
+      </c>
+      <c r="G218" s="11" t="inlineStr">
+        <is>
+          <t>Partial — pair with Claude to draft campaigns</t>
+        </is>
+      </c>
+      <c r="H218" s="11" t="inlineStr">
+        <is>
+          <t>Free at any scale; fast; API-driven</t>
+        </is>
+      </c>
+      <c r="I218" s="11" t="inlineStr">
+        <is>
+          <t>Warm-list campaigns, not cold outreach</t>
+        </is>
+      </c>
+      <c r="J218" s="11" t="inlineStr">
+        <is>
+          <t>Self-hosters sending email campaigns</t>
+        </is>
+      </c>
+      <c r="K218" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="L218" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="M218" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N218" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="O218" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219" ht="22" customHeight="1">
+      <c r="A219" s="4" t="inlineStr">
+        <is>
+          <t>AI Marketing &amp; SEO</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" ht="58" customHeight="1">
+      <c r="A220" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=semrush.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B220" s="6" t="inlineStr">
+        <is>
+          <t>Semrush</t>
+        </is>
+      </c>
+      <c r="C220" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D220" s="8" t="inlineStr">
+        <is>
+          <t>semrush.com</t>
+        </is>
+      </c>
+      <c r="E220" s="7" t="inlineStr">
+        <is>
+          <t>All-in-one SEO/SEM platform with AI features and ContentShake</t>
+        </is>
+      </c>
+      <c r="F220" s="7" t="inlineStr">
+        <is>
+          <t>From $139.95/mo</t>
+        </is>
+      </c>
+      <c r="G220" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H220" s="7" t="inlineStr">
+        <is>
+          <t>Deepest SEO dataset; AI content tools</t>
+        </is>
+      </c>
+      <c r="I220" s="7" t="inlineStr">
+        <is>
+          <t>Expensive; overwhelming</t>
+        </is>
+      </c>
+      <c r="J220" s="7" t="inlineStr">
+        <is>
+          <t>SEO professionals</t>
+        </is>
+      </c>
+      <c r="K220" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L220" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M220" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="N220" s="5" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="O220" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="221" ht="58" customHeight="1">
+      <c r="A221" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=ahrefs.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B221" s="6" t="inlineStr">
+        <is>
+          <t>Ahrefs</t>
+        </is>
+      </c>
+      <c r="C221" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D221" s="8" t="inlineStr">
+        <is>
+          <t>ahrefs.com</t>
+        </is>
+      </c>
+      <c r="E221" s="7" t="inlineStr">
+        <is>
+          <t>Backlink/keyword research leader with AI content helper</t>
+        </is>
+      </c>
+      <c r="F221" s="7" t="inlineStr">
+        <is>
+          <t>From $129/mo</t>
+        </is>
+      </c>
+      <c r="G221" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H221" s="7" t="inlineStr">
+        <is>
+          <t>Best link data; clean UX</t>
+        </is>
+      </c>
+      <c r="I221" s="7" t="inlineStr">
+        <is>
+          <t>No free tier; AI is light</t>
+        </is>
+      </c>
+      <c r="J221" s="7" t="inlineStr">
+        <is>
+          <t>Link-building and SEO research</t>
+        </is>
+      </c>
+      <c r="K221" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L221" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M221" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="N221" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="O221" s="5" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="222" ht="58" customHeight="1">
+      <c r="A222" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=surferseo.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B222" s="6" t="inlineStr">
+        <is>
+          <t>Surfer</t>
+        </is>
+      </c>
+      <c r="C222" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D222" s="8" t="inlineStr">
+        <is>
+          <t>surferseo.com</t>
+        </is>
+      </c>
+      <c r="E222" s="7" t="inlineStr">
+        <is>
+          <t>On-page SEO content optimisation with AI writing</t>
+        </is>
+      </c>
+      <c r="F222" s="7" t="inlineStr">
+        <is>
+          <t>From $89/mo</t>
+        </is>
+      </c>
+      <c r="G222" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H222" s="7" t="inlineStr">
+        <is>
+          <t>Clear data-driven content scores</t>
+        </is>
+      </c>
+      <c r="I222" s="7" t="inlineStr">
+        <is>
+          <t>Per-article economics; SERP-chasing risk</t>
+        </is>
+      </c>
+      <c r="J222" s="7" t="inlineStr">
+        <is>
+          <t>Content teams optimising for Google</t>
+        </is>
+      </c>
+      <c r="K222" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L222" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="M222" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="N222" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="O222" s="5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="223" ht="58" customHeight="1">
+      <c r="A223" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=adcreative.ai&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B223" s="6" t="inlineStr">
+        <is>
+          <t>AdCreative.ai</t>
+        </is>
+      </c>
+      <c r="C223" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D223" s="8" t="inlineStr">
+        <is>
+          <t>adcreative.ai</t>
+        </is>
+      </c>
+      <c r="E223" s="7" t="inlineStr">
+        <is>
+          <t>AI ad creative and copy generation with performance scoring</t>
+        </is>
+      </c>
+      <c r="F223" s="7" t="inlineStr">
+        <is>
+          <t>From $25/mo</t>
+        </is>
+      </c>
+      <c r="G223" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H223" s="7" t="inlineStr">
+        <is>
+          <t>Volume ad-variant generation; scoring</t>
+        </is>
+      </c>
+      <c r="I223" s="7" t="inlineStr">
+        <is>
+          <t>Template look; aggressive billing reputation — check terms</t>
+        </is>
+      </c>
+      <c r="J223" s="7" t="inlineStr">
+        <is>
+          <t>Performance marketers</t>
+        </is>
+      </c>
+      <c r="K223" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L223" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M223" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N223" s="5" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="O223" s="5" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="224" ht="58" customHeight="1">
+      <c r="A224" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=hootsuite.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B224" s="6" t="inlineStr">
+        <is>
+          <t>Hootsuite</t>
+        </is>
+      </c>
+      <c r="C224" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D224" s="8" t="inlineStr">
+        <is>
+          <t>hootsuite.com</t>
+        </is>
+      </c>
+      <c r="E224" s="7" t="inlineStr">
+        <is>
+          <t>Social media management with OwlyWriter AI</t>
+        </is>
+      </c>
+      <c r="F224" s="7" t="inlineStr">
+        <is>
+          <t>From $99/mo</t>
+        </is>
+      </c>
+      <c r="G224" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H224" s="7" t="inlineStr">
+        <is>
+          <t>Mature scheduling/listening suite</t>
+        </is>
+      </c>
+      <c r="I224" s="7" t="inlineStr">
+        <is>
+          <t>Expensive; AI basic</t>
+        </is>
+      </c>
+      <c r="J224" s="7" t="inlineStr">
+        <is>
+          <t>Social teams managing many accounts</t>
+        </is>
+      </c>
+      <c r="K224" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L224" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M224" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N224" s="5" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="O224" s="5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="225" ht="58" customHeight="1">
+      <c r="A225" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=buffer.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B225" s="6" t="inlineStr">
+        <is>
+          <t>Buffer</t>
+        </is>
+      </c>
+      <c r="C225" s="7" t="inlineStr">
+        <is>
+          <t>Freemium</t>
+        </is>
+      </c>
+      <c r="D225" s="8" t="inlineStr">
+        <is>
+          <t>buffer.com</t>
+        </is>
+      </c>
+      <c r="E225" s="7" t="inlineStr">
+        <is>
+          <t>Simple social scheduling with AI assistant</t>
+        </is>
+      </c>
+      <c r="F225" s="7" t="inlineStr">
+        <is>
+          <t>Free; $6/channel/mo</t>
+        </is>
+      </c>
+      <c r="G225" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H225" s="7" t="inlineStr">
+        <is>
+          <t>Affordable; clean; good AI repurposing</t>
+        </is>
+      </c>
+      <c r="I225" s="7" t="inlineStr">
+        <is>
+          <t>Lighter analytics</t>
+        </is>
+      </c>
+      <c r="J225" s="7" t="inlineStr">
+        <is>
+          <t>Creators and small brands</t>
+        </is>
+      </c>
+      <c r="K225" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L225" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="M225" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N225" s="5" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="O225" s="5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="226" ht="58" customHeight="1">
+      <c r="A226" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=mailchimp.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B226" s="6" t="inlineStr">
+        <is>
+          <t>Mailchimp</t>
+        </is>
+      </c>
+      <c r="C226" s="7" t="inlineStr">
+        <is>
+          <t>Freemium</t>
+        </is>
+      </c>
+      <c r="D226" s="8" t="inlineStr">
+        <is>
+          <t>mailchimp.com</t>
+        </is>
+      </c>
+      <c r="E226" s="7" t="inlineStr">
+        <is>
+          <t>Email marketing with AI content and journeys</t>
+        </is>
+      </c>
+      <c r="F226" s="7" t="inlineStr">
+        <is>
+          <t>Free; from $13/mo</t>
+        </is>
+      </c>
+      <c r="G226" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H226" s="7" t="inlineStr">
+        <is>
+          <t>Familiar; AI campaign generation</t>
+        </is>
+      </c>
+      <c r="I226" s="7" t="inlineStr">
+        <is>
+          <t>Pricing grows with list; CRM-lite</t>
+        </is>
+      </c>
+      <c r="J226" s="7" t="inlineStr">
+        <is>
+          <t>SMB email marketing</t>
+        </is>
+      </c>
+      <c r="K226" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L226" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M226" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N226" s="5" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="O226" s="5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="227" ht="58" customHeight="1">
+      <c r="A227" s="9">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B227" s="10" t="inlineStr">
+        <is>
+          <t>Mautic</t>
+        </is>
+      </c>
+      <c r="C227" s="11" t="inlineStr">
+        <is>
+          <t>Open source (GitHub)</t>
+        </is>
+      </c>
+      <c r="D227" s="12" t="inlineStr">
+        <is>
+          <t>github.com/mautic/mautic</t>
+        </is>
+      </c>
+      <c r="E227" s="11" t="inlineStr">
+        <is>
+          <t>Open-source marketing automation (email, journeys, segmentation)</t>
+        </is>
+      </c>
+      <c r="F227" s="11" t="inlineStr">
+        <is>
+          <t>Free (self-host)</t>
+        </is>
+      </c>
+      <c r="G227" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H227" s="11" t="inlineStr">
+        <is>
+          <t>Full marketing automation without per-contact fees</t>
+        </is>
+      </c>
+      <c r="I227" s="11" t="inlineStr">
+        <is>
+          <t>Self-host complexity; plugins needed</t>
+        </is>
+      </c>
+      <c r="J227" s="11" t="inlineStr">
+        <is>
+          <t>Companies escaping HubSpot/Marketo pricing</t>
+        </is>
+      </c>
+      <c r="K227" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="L227" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="M227" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="N227" s="9" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="O227" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228" ht="58" customHeight="1">
+      <c r="A228" s="9">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B228" s="10" t="inlineStr">
+        <is>
+          <t>Postiz</t>
+        </is>
+      </c>
+      <c r="C228" s="11" t="inlineStr">
+        <is>
+          <t>Open source (GitHub)</t>
+        </is>
+      </c>
+      <c r="D228" s="12" t="inlineStr">
+        <is>
+          <t>github.com/gitroomhq/postiz-app</t>
+        </is>
+      </c>
+      <c r="E228" s="11" t="inlineStr">
+        <is>
+          <t>Open-source AI social media scheduling (Buffer/Hootsuite alternative)</t>
+        </is>
+      </c>
+      <c r="F228" s="11" t="inlineStr">
+        <is>
+          <t>Free self-host; cloud from $29/mo</t>
+        </is>
+      </c>
+      <c r="G228" s="11" t="inlineStr">
+        <is>
+          <t>Partial — BYO AI keys</t>
+        </is>
+      </c>
+      <c r="H228" s="11" t="inlineStr">
+        <is>
+          <t>OSS scheduling for 15+ platforms with AI</t>
+        </is>
+      </c>
+      <c r="I228" s="11" t="inlineStr">
+        <is>
+          <t>Young project</t>
+        </is>
+      </c>
+      <c r="J228" s="11" t="inlineStr">
+        <is>
+          <t>Self-hosted social scheduling</t>
+        </is>
+      </c>
+      <c r="K228" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L228" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="M228" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N228" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="O228" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="229" ht="58" customHeight="1">
+      <c r="A229" s="9">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B229" s="10" t="inlineStr">
+        <is>
+          <t>Matomo</t>
+        </is>
+      </c>
+      <c r="C229" s="11" t="inlineStr">
+        <is>
+          <t>Open source (GitHub)</t>
+        </is>
+      </c>
+      <c r="D229" s="12" t="inlineStr">
+        <is>
+          <t>github.com/matomo-org/matomo</t>
+        </is>
+      </c>
+      <c r="E229" s="11" t="inlineStr">
+        <is>
+          <t>Open-source web analytics (Google Analytics alternative)</t>
+        </is>
+      </c>
+      <c r="F229" s="11" t="inlineStr">
+        <is>
+          <t>Free self-host; cloud from $23/mo</t>
+        </is>
+      </c>
+      <c r="G229" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H229" s="11" t="inlineStr">
+        <is>
+          <t>Privacy-compliant analytics you own</t>
+        </is>
+      </c>
+      <c r="I229" s="11" t="inlineStr">
+        <is>
+          <t>No AI insights layer yet</t>
+        </is>
+      </c>
+      <c r="J229" s="11" t="inlineStr">
+        <is>
+          <t>Privacy-first site analytics</t>
+        </is>
+      </c>
+      <c r="K229" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L229" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="M229" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="N229" s="9" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="O229" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="230" ht="22" customHeight="1">
+      <c r="A230" s="4" t="inlineStr">
+        <is>
+          <t>AI Research Tools</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="58" customHeight="1">
+      <c r="A231" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=elicit.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B231" s="6" t="inlineStr">
+        <is>
+          <t>Elicit</t>
+        </is>
+      </c>
+      <c r="C231" s="7" t="inlineStr">
+        <is>
+          <t>Freemium</t>
+        </is>
+      </c>
+      <c r="D231" s="8" t="inlineStr">
+        <is>
+          <t>elicit.com</t>
+        </is>
+      </c>
+      <c r="E231" s="7" t="inlineStr">
+        <is>
+          <t>AI research assistant that searches and summarises academic papers</t>
+        </is>
+      </c>
+      <c r="F231" s="7" t="inlineStr">
+        <is>
+          <t>Free; Plus $12/mo</t>
+        </is>
+      </c>
+      <c r="G231" s="7" t="inlineStr">
+        <is>
+          <t>No — (Anthropic models used under the hood historically)</t>
+        </is>
+      </c>
+      <c r="H231" s="7" t="inlineStr">
+        <is>
+          <t>Systematic-review-grade extraction tables</t>
+        </is>
+      </c>
+      <c r="I231" s="7" t="inlineStr">
+        <is>
+          <t>Academic papers only</t>
+        </is>
+      </c>
+      <c r="J231" s="7" t="inlineStr">
+        <is>
+          <t>Researchers and grad students</t>
+        </is>
+      </c>
+      <c r="K231" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L231" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="M231" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="N231" s="5" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="O231" s="5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="232" ht="58" customHeight="1">
+      <c r="A232" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=consensus.app&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B232" s="6" t="inlineStr">
+        <is>
+          <t>Consensus</t>
+        </is>
+      </c>
+      <c r="C232" s="7" t="inlineStr">
+        <is>
+          <t>Freemium</t>
+        </is>
+      </c>
+      <c r="D232" s="8" t="inlineStr">
+        <is>
+          <t>consensus.app</t>
+        </is>
+      </c>
+      <c r="E232" s="7" t="inlineStr">
+        <is>
+          <t>Search engine answering questions from peer-reviewed evidence</t>
+        </is>
+      </c>
+      <c r="F232" s="7" t="inlineStr">
+        <is>
+          <t>Free; Premium $11.99/mo</t>
+        </is>
+      </c>
+      <c r="G232" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H232" s="7" t="inlineStr">
+        <is>
+          <t>Evidence meters; citation-grounded answers</t>
+        </is>
+      </c>
+      <c r="I232" s="7" t="inlineStr">
+        <is>
+          <t>Narrower than general search</t>
+        </is>
+      </c>
+      <c r="J232" s="7" t="inlineStr">
+        <is>
+          <t>Evidence-based professionals</t>
+        </is>
+      </c>
+      <c r="K232" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L232" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="M232" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N232" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="O232" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="233" ht="58" customHeight="1">
+      <c r="A233" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=scispace.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B233" s="6" t="inlineStr">
+        <is>
+          <t>SciSpace</t>
+        </is>
+      </c>
+      <c r="C233" s="7" t="inlineStr">
+        <is>
+          <t>Freemium</t>
+        </is>
+      </c>
+      <c r="D233" s="8" t="inlineStr">
+        <is>
+          <t>scispace.com</t>
+        </is>
+      </c>
+      <c r="E233" s="7" t="inlineStr">
+        <is>
+          <t>Read, annotate and chat with research PDFs; literature review AI</t>
+        </is>
+      </c>
+      <c r="F233" s="7" t="inlineStr">
+        <is>
+          <t>Free; from $12/mo</t>
+        </is>
+      </c>
+      <c r="G233" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H233" s="7" t="inlineStr">
+        <is>
+          <t>Great PDF explanation UX</t>
+        </is>
+      </c>
+      <c r="I233" s="7" t="inlineStr">
+        <is>
+          <t>Aggressive upsells</t>
+        </is>
+      </c>
+      <c r="J233" s="7" t="inlineStr">
+        <is>
+          <t>Students decoding dense papers</t>
+        </is>
+      </c>
+      <c r="K233" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L233" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="M233" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N233" s="5" t="n">
         <v>5.7</v>
       </c>
-      <c r="O213" s="5" t="n">
+      <c r="O233" s="5" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="214" ht="58" customHeight="1">
-      <c r="A214" s="9">
+    <row r="234" ht="58" customHeight="1">
+      <c r="A234" s="9">
         <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
         <v/>
       </c>
-      <c r="B214" s="10" t="inlineStr">
+      <c r="B234" s="10" t="inlineStr">
         <is>
           <t>GPT Researcher</t>
         </is>
       </c>
-      <c r="C214" s="11" t="inlineStr">
+      <c r="C234" s="11" t="inlineStr">
         <is>
           <t>Open source (GitHub)</t>
         </is>
       </c>
-      <c r="D214" s="12" t="inlineStr">
+      <c r="D234" s="12" t="inlineStr">
         <is>
           <t>github.com/assafelovic/gpt-researcher</t>
         </is>
       </c>
-      <c r="E214" s="11" t="inlineStr">
+      <c r="E234" s="11" t="inlineStr">
         <is>
           <t>Open-source autonomous deep-research agent producing cited reports</t>
         </is>
       </c>
-      <c r="F214" s="11" t="inlineStr">
+      <c r="F234" s="11" t="inlineStr">
         <is>
           <t>Free + API costs</t>
         </is>
       </c>
-      <c r="G214" s="11" t="inlineStr">
+      <c r="G234" s="11" t="inlineStr">
         <is>
           <t>Yes — supports Anthropic/Claude as the LLM</t>
         </is>
       </c>
-      <c r="H214" s="11" t="inlineStr">
+      <c r="H234" s="11" t="inlineStr">
         <is>
           <t>Free deep-research with citations; local &amp; web</t>
         </is>
       </c>
-      <c r="I214" s="11" t="inlineStr">
+      <c r="I234" s="11" t="inlineStr">
         <is>
           <t>Setup + API keys; report quality varies by model</t>
         </is>
       </c>
-      <c r="J214" s="11" t="inlineStr">
+      <c r="J234" s="11" t="inlineStr">
         <is>
           <t>Developers automating research</t>
         </is>
       </c>
-      <c r="K214" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="L214" s="9" t="n">
+      <c r="K234" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="L234" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="M214" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="N214" s="9" t="n">
+      <c r="M234" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="N234" s="9" t="n">
         <v>7.7</v>
       </c>
-      <c r="O214" s="9" t="n">
+      <c r="O234" s="9" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="215" ht="58" customHeight="1">
-      <c r="A215" s="9">
+    <row r="235" ht="58" customHeight="1">
+      <c r="A235" s="9">
         <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
         <v/>
       </c>
-      <c r="B215" s="10" t="inlineStr">
+      <c r="B235" s="10" t="inlineStr">
         <is>
           <t>STORM</t>
         </is>
       </c>
-      <c r="C215" s="11" t="inlineStr">
+      <c r="C235" s="11" t="inlineStr">
         <is>
           <t>Open source (GitHub)</t>
         </is>
       </c>
-      <c r="D215" s="12" t="inlineStr">
+      <c r="D235" s="12" t="inlineStr">
         <is>
           <t>github.com/stanford-oval/storm</t>
         </is>
       </c>
-      <c r="E215" s="11" t="inlineStr">
+      <c r="E235" s="11" t="inlineStr">
         <is>
           <t>Stanford's open-source Wikipedia-style article research/writing system</t>
         </is>
       </c>
-      <c r="F215" s="11" t="inlineStr">
+      <c r="F235" s="11" t="inlineStr">
         <is>
           <t>Free + API costs</t>
         </is>
       </c>
-      <c r="G215" s="11" t="inlineStr">
+      <c r="G235" s="11" t="inlineStr">
         <is>
           <t>Yes — configurable to Claude models</t>
         </is>
       </c>
-      <c r="H215" s="11" t="inlineStr">
+      <c r="H235" s="11" t="inlineStr">
         <is>
           <t>Research-grade outline→article pipeline</t>
         </is>
       </c>
-      <c r="I215" s="11" t="inlineStr">
+      <c r="I235" s="11" t="inlineStr">
         <is>
           <t>Academic tool; rough edges</t>
         </is>
       </c>
-      <c r="J215" s="11" t="inlineStr">
+      <c r="J235" s="11" t="inlineStr">
         <is>
           <t>Long-form grounded content experiments</t>
         </is>
       </c>
-      <c r="K215" s="9" t="n">
+      <c r="K235" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="L215" s="9" t="n">
+      <c r="L235" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="M215" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N215" s="9" t="n">
+      <c r="M235" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N235" s="9" t="n">
         <v>6.7</v>
       </c>
-      <c r="O215" s="9" t="n">
+      <c r="O235" s="9" t="n">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
+    <mergeCell ref="A78:O78"/>
+    <mergeCell ref="A164:O164"/>
+    <mergeCell ref="A46:O46"/>
+    <mergeCell ref="A101:O101"/>
+    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A175:O175"/>
+    <mergeCell ref="A203:O203"/>
+    <mergeCell ref="A188:O188"/>
+    <mergeCell ref="A135:O135"/>
+    <mergeCell ref="A219:O219"/>
+    <mergeCell ref="A122:O122"/>
+    <mergeCell ref="A112:O112"/>
+    <mergeCell ref="A230:O230"/>
+    <mergeCell ref="A34:O34"/>
+    <mergeCell ref="A143:O143"/>
     <mergeCell ref="A15:O15"/>
     <mergeCell ref="A59:O59"/>
-    <mergeCell ref="A135:O135"/>
+    <mergeCell ref="A88:O88"/>
     <mergeCell ref="A153:O153"/>
-    <mergeCell ref="A2:O2"/>
-    <mergeCell ref="A101:O101"/>
-    <mergeCell ref="A210:O210"/>
-    <mergeCell ref="A175:O175"/>
-    <mergeCell ref="A112:O112"/>
-    <mergeCell ref="A199:O199"/>
-    <mergeCell ref="A164:O164"/>
-    <mergeCell ref="A46:O46"/>
-    <mergeCell ref="A188:O188"/>
-    <mergeCell ref="A88:O88"/>
-    <mergeCell ref="A34:O34"/>
-    <mergeCell ref="A143:O143"/>
-    <mergeCell ref="A78:O78"/>
-    <mergeCell ref="A122:O122"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
@@ -14041,21 +15303,40 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D196" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D197" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D198" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D200" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D201" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D202" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D203" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D199" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D200" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D201" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D202" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D204" r:id="rId186"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D205" r:id="rId187"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D206" r:id="rId188"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D207" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D208" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D209" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D212" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D213" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D214" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D215" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D210" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D212" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D213" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D214" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D215" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D216" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D217" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D218" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D220" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D221" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D222" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D223" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D224" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D225" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D226" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D227" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D228" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D229" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D231" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D232" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D233" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D234" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D235" r:id="rId215"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14067,7 +15348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -14527,7 +15808,7 @@
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Salesforce (Agentforce)</t>
         </is>
       </c>
       <c r="E17" s="16" t="inlineStr">
@@ -14539,52 +15820,79 @@
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>AI Marketing &amp; SEO</t>
+          <t>AI Sales Outreach &amp; Prospecting</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>Mautic</t>
+          <t>Listmonk</t>
         </is>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>Postiz</t>
+          <t>Instantly</t>
         </is>
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>Matomo</t>
+          <t>Smartlead</t>
         </is>
       </c>
       <c r="E18" s="16" t="inlineStr">
         <is>
-          <t>Mautic</t>
+          <t>Listmonk</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
+          <t>AI Marketing &amp; SEO</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>Mautic</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Postiz</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>Matomo</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>Mautic</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
           <t>AI Research Tools</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>GPT Researcher</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>Elicit</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>STORM</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E20" s="16" t="inlineStr">
         <is>
           <t>GPT Researcher</t>
         </is>

</xml_diff>

<commit_message>
Add Blueticks (WhatsApp scheduler, campaigns, AI agent & CRM) to AI Sales & CRM
Blueticks is a WhatsApp automation Chrome extension (scheduler, bulk
marketing campaigns, AI support agent, CRM/task management) that ships an
official MCP server letting Claude read, send and schedule WhatsApp
messages. Regenerated all spreadsheet/CSV outputs (now 231 tools).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRaLc5h85fXAmfthxHaxVx
</commit_message>
<xml_diff>
--- a/AI-Tools-Directory.xlsx
+++ b/AI-Tools-Directory.xlsx
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O250"/>
+  <dimension ref="A1:O251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -12699,7 +12699,7 @@
         <v>6.7</v>
       </c>
       <c r="O196" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="197" ht="58" customHeight="1">
@@ -12765,7 +12765,7 @@
         <v>6.3</v>
       </c>
       <c r="O197" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="198" ht="58" customHeight="1">
@@ -12831,7 +12831,7 @@
         <v>5.7</v>
       </c>
       <c r="O198" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="199" ht="58" customHeight="1">
@@ -12897,7 +12897,7 @@
         <v>5.7</v>
       </c>
       <c r="O199" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="200" ht="58" customHeight="1">
@@ -12963,7 +12963,7 @@
         <v>5.3</v>
       </c>
       <c r="O200" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="201" ht="58" customHeight="1">
@@ -13029,7 +13029,7 @@
         <v>6</v>
       </c>
       <c r="O201" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="202" ht="58" customHeight="1">
@@ -13095,7 +13095,7 @@
         <v>5.7</v>
       </c>
       <c r="O202" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="203" ht="58" customHeight="1">
@@ -13161,73 +13161,73 @@
         <v>5.7</v>
       </c>
       <c r="O203" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="204" ht="58" customHeight="1">
-      <c r="A204" s="9">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B204" s="10" t="inlineStr">
-        <is>
-          <t>Twenty</t>
-        </is>
-      </c>
-      <c r="C204" s="11" t="inlineStr">
-        <is>
-          <t>Open source (GitHub)</t>
-        </is>
-      </c>
-      <c r="D204" s="12" t="inlineStr">
-        <is>
-          <t>github.com/twentyhq/twenty</t>
-        </is>
-      </c>
-      <c r="E204" s="11" t="inlineStr">
-        <is>
-          <t>Modern open-source CRM (the OSS Salesforce alternative)</t>
-        </is>
-      </c>
-      <c r="F204" s="11" t="inlineStr">
-        <is>
-          <t>Free self-host; cloud from $9/user/mo</t>
-        </is>
-      </c>
-      <c r="G204" s="11" t="inlineStr">
-        <is>
-          <t>Partial — API/webhooks; community MCP</t>
-        </is>
-      </c>
-      <c r="H204" s="11" t="inlineStr">
-        <is>
-          <t>Beautiful modern OSS CRM; data ownership</t>
-        </is>
-      </c>
-      <c r="I204" s="11" t="inlineStr">
-        <is>
-          <t>Younger ecosystem; fewer native integrations</t>
-        </is>
-      </c>
-      <c r="J204" s="11" t="inlineStr">
-        <is>
-          <t>Startups wanting an ownable CRM</t>
-        </is>
-      </c>
-      <c r="K204" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="L204" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="M204" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="N204" s="9" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="O204" s="9" t="n">
-        <v>2</v>
+      <c r="A204" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=blueticks.co&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B204" s="6" t="inlineStr">
+        <is>
+          <t>Blueticks</t>
+        </is>
+      </c>
+      <c r="C204" s="7" t="inlineStr">
+        <is>
+          <t>Freemium</t>
+        </is>
+      </c>
+      <c r="D204" s="8" t="inlineStr">
+        <is>
+          <t>blueticks.co</t>
+        </is>
+      </c>
+      <c r="E204" s="7" t="inlineStr">
+        <is>
+          <t>WhatsApp scheduler, bulk marketing campaigns, AI support agent and CRM/task management (Chrome extension)</t>
+        </is>
+      </c>
+      <c r="F204" s="7" t="inlineStr">
+        <is>
+          <t>Free (1 msg at a time); paid from ~$15/mo</t>
+        </is>
+      </c>
+      <c r="G204" s="7" t="inlineStr">
+        <is>
+          <t>Yes — official Blueticks MCP server lets Claude read, send and schedule WhatsApp messages</t>
+        </is>
+      </c>
+      <c r="H204" s="7" t="inlineStr">
+        <is>
+          <t>Botless WhatsApp automation from your own number; MCP lets Claude operate WhatsApp; privacy-first (data stays on device)</t>
+        </is>
+      </c>
+      <c r="I204" s="7" t="inlineStr">
+        <is>
+          <t>Unofficial WhatsApp automation risks account limits; Chrome-extension-bound; not affiliated with Meta</t>
+        </is>
+      </c>
+      <c r="J204" s="7" t="inlineStr">
+        <is>
+          <t>SMBs and sellers running sales &amp; support over WhatsApp</t>
+        </is>
+      </c>
+      <c r="K204" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="L204" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="M204" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N204" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="O204" s="5" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="205" ht="58" customHeight="1">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="B205" s="10" t="inlineStr">
         <is>
-          <t>EspoCRM</t>
+          <t>Twenty</t>
         </is>
       </c>
       <c r="C205" s="11" t="inlineStr">
@@ -13247,53 +13247,53 @@
       </c>
       <c r="D205" s="12" t="inlineStr">
         <is>
-          <t>github.com/espocrm/espocrm</t>
+          <t>github.com/twentyhq/twenty</t>
         </is>
       </c>
       <c r="E205" s="11" t="inlineStr">
         <is>
-          <t>Mature open-source CRM with workflows and email</t>
+          <t>Modern open-source CRM (the OSS Salesforce alternative)</t>
         </is>
       </c>
       <c r="F205" s="11" t="inlineStr">
         <is>
-          <t>Free self-host; cloud from $15/mo</t>
+          <t>Free self-host; cloud from $9/user/mo</t>
         </is>
       </c>
       <c r="G205" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partial — API/webhooks; community MCP</t>
         </is>
       </c>
       <c r="H205" s="11" t="inlineStr">
         <is>
-          <t>Proven, full-featured, cheap</t>
+          <t>Beautiful modern OSS CRM; data ownership</t>
         </is>
       </c>
       <c r="I205" s="11" t="inlineStr">
         <is>
-          <t>Dated UI; AI minimal</t>
+          <t>Younger ecosystem; fewer native integrations</t>
         </is>
       </c>
       <c r="J205" s="11" t="inlineStr">
         <is>
-          <t>Cost-sensitive sales teams</t>
+          <t>Startups wanting an ownable CRM</t>
         </is>
       </c>
       <c r="K205" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L205" s="9" t="n">
         <v>10</v>
       </c>
       <c r="M205" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N205" s="9" t="n">
-        <v>6.7</v>
+        <v>7.7</v>
       </c>
       <c r="O205" s="9" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="206" ht="58" customHeight="1">
@@ -13303,7 +13303,7 @@
       </c>
       <c r="B206" s="10" t="inlineStr">
         <is>
-          <t>Frappe CRM</t>
+          <t>EspoCRM</t>
         </is>
       </c>
       <c r="C206" s="11" t="inlineStr">
@@ -13313,17 +13313,17 @@
       </c>
       <c r="D206" s="12" t="inlineStr">
         <is>
-          <t>github.com/frappe/crm</t>
+          <t>github.com/espocrm/espocrm</t>
         </is>
       </c>
       <c r="E206" s="11" t="inlineStr">
         <is>
-          <t>Clean open-source CRM from the ERPNext ecosystem</t>
+          <t>Mature open-source CRM with workflows and email</t>
         </is>
       </c>
       <c r="F206" s="11" t="inlineStr">
         <is>
-          <t>Free self-host; cloud plans</t>
+          <t>Free self-host; cloud from $15/mo</t>
         </is>
       </c>
       <c r="G206" s="11" t="inlineStr">
@@ -13333,17 +13333,17 @@
       </c>
       <c r="H206" s="11" t="inlineStr">
         <is>
-          <t>Modern UX; ERPNext integration</t>
+          <t>Proven, full-featured, cheap</t>
         </is>
       </c>
       <c r="I206" s="11" t="inlineStr">
         <is>
-          <t>Smaller community</t>
+          <t>Dated UI; AI minimal</t>
         </is>
       </c>
       <c r="J206" s="11" t="inlineStr">
         <is>
-          <t>Companies already on Frappe/ERPNext</t>
+          <t>Cost-sensitive sales teams</t>
         </is>
       </c>
       <c r="K206" s="9" t="n">
@@ -13353,116 +13353,116 @@
         <v>10</v>
       </c>
       <c r="M206" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N206" s="9" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="O206" s="9" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="207" ht="58" customHeight="1">
+      <c r="A207" s="9">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B207" s="10" t="inlineStr">
+        <is>
+          <t>Frappe CRM</t>
+        </is>
+      </c>
+      <c r="C207" s="11" t="inlineStr">
+        <is>
+          <t>Open source (GitHub)</t>
+        </is>
+      </c>
+      <c r="D207" s="12" t="inlineStr">
+        <is>
+          <t>github.com/frappe/crm</t>
+        </is>
+      </c>
+      <c r="E207" s="11" t="inlineStr">
+        <is>
+          <t>Clean open-source CRM from the ERPNext ecosystem</t>
+        </is>
+      </c>
+      <c r="F207" s="11" t="inlineStr">
+        <is>
+          <t>Free self-host; cloud plans</t>
+        </is>
+      </c>
+      <c r="G207" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H207" s="11" t="inlineStr">
+        <is>
+          <t>Modern UX; ERPNext integration</t>
+        </is>
+      </c>
+      <c r="I207" s="11" t="inlineStr">
+        <is>
+          <t>Smaller community</t>
+        </is>
+      </c>
+      <c r="J207" s="11" t="inlineStr">
+        <is>
+          <t>Companies already on Frappe/ERPNext</t>
+        </is>
+      </c>
+      <c r="K207" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L207" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="M207" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="N206" s="9" t="n">
+      <c r="N207" s="9" t="n">
         <v>6.3</v>
       </c>
-      <c r="O206" s="9" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="207" ht="22" customHeight="1">
-      <c r="A207" s="4" t="inlineStr">
+      <c r="O207" s="9" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="208" ht="22" customHeight="1">
+      <c r="A208" s="4" t="inlineStr">
         <is>
           <t>AI Sales Outreach &amp; Prospecting</t>
         </is>
-      </c>
-    </row>
-    <row r="208" ht="58" customHeight="1">
-      <c r="A208" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=zoominfo.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B208" s="6" t="inlineStr">
-        <is>
-          <t>ZoomInfo Copilot</t>
-        </is>
-      </c>
-      <c r="C208" s="7" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="D208" s="8" t="inlineStr">
-        <is>
-          <t>zoominfo.com</t>
-        </is>
-      </c>
-      <c r="E208" s="7" t="inlineStr">
-        <is>
-          <t>B2B contact/company database with intent data and an AI copilot</t>
-        </is>
-      </c>
-      <c r="F208" s="7" t="inlineStr">
-        <is>
-          <t>From ~$15k/yr (contract)</t>
-        </is>
-      </c>
-      <c r="G208" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H208" s="7" t="inlineStr">
-        <is>
-          <t>Deepest B2B data + buying-intent signals</t>
-        </is>
-      </c>
-      <c r="I208" s="7" t="inlineStr">
-        <is>
-          <t>Expensive annual contracts</t>
-        </is>
-      </c>
-      <c r="J208" s="7" t="inlineStr">
-        <is>
-          <t>Enterprise outbound teams</t>
-        </is>
-      </c>
-      <c r="K208" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="L208" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="M208" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="N208" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="O208" s="5" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="209" ht="58" customHeight="1">
       <c r="A209" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=lusha.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=zoominfo.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B209" s="6" t="inlineStr">
         <is>
-          <t>Lusha</t>
+          <t>ZoomInfo Copilot</t>
         </is>
       </c>
       <c r="C209" s="7" t="inlineStr">
         <is>
-          <t>Freemium</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="D209" s="8" t="inlineStr">
         <is>
-          <t>lusha.com</t>
+          <t>zoominfo.com</t>
         </is>
       </c>
       <c r="E209" s="7" t="inlineStr">
         <is>
-          <t>B2B contact data via web app and Chrome extension</t>
+          <t>B2B contact/company database with intent data and an AI copilot</t>
         </is>
       </c>
       <c r="F209" s="7" t="inlineStr">
         <is>
-          <t>Free; from $36/user/mo</t>
+          <t>From ~$15k/yr (contract)</t>
         </is>
       </c>
       <c r="G209" s="7" t="inlineStr">
@@ -13472,43 +13472,43 @@
       </c>
       <c r="H209" s="7" t="inlineStr">
         <is>
-          <t>Easy to use; compliance-focused data</t>
+          <t>Deepest B2B data + buying-intent signals</t>
         </is>
       </c>
       <c r="I209" s="7" t="inlineStr">
         <is>
-          <t>Smaller database than ZoomInfo</t>
+          <t>Expensive annual contracts</t>
         </is>
       </c>
       <c r="J209" s="7" t="inlineStr">
         <is>
-          <t>SDRs needing quick contact data</t>
+          <t>Enterprise outbound teams</t>
         </is>
       </c>
       <c r="K209" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L209" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M209" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="N209" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="O209" s="5" t="n">
         <v>5</v>
-      </c>
-      <c r="L209" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="M209" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N209" s="5" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="O209" s="5" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="210" ht="58" customHeight="1">
       <c r="A210" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=seamless.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=lusha.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B210" s="6" t="inlineStr">
         <is>
-          <t>Seamless.AI</t>
+          <t>Lusha</t>
         </is>
       </c>
       <c r="C210" s="7" t="inlineStr">
@@ -13518,17 +13518,17 @@
       </c>
       <c r="D210" s="8" t="inlineStr">
         <is>
-          <t>seamless.ai</t>
+          <t>lusha.com</t>
         </is>
       </c>
       <c r="E210" s="7" t="inlineStr">
         <is>
-          <t>Real-time AI search engine for B2B contact information</t>
+          <t>B2B contact data via web app and Chrome extension</t>
         </is>
       </c>
       <c r="F210" s="7" t="inlineStr">
         <is>
-          <t>Free credits; from ~$147/mo</t>
+          <t>Free; from $36/user/mo</t>
         </is>
       </c>
       <c r="G210" s="7" t="inlineStr">
@@ -13538,63 +13538,63 @@
       </c>
       <c r="H210" s="7" t="inlineStr">
         <is>
-          <t>Real-time verification; high volumes</t>
+          <t>Easy to use; compliance-focused data</t>
         </is>
       </c>
       <c r="I210" s="7" t="inlineStr">
         <is>
-          <t>Data-accuracy complaints; pushy sales motion</t>
+          <t>Smaller database than ZoomInfo</t>
         </is>
       </c>
       <c r="J210" s="7" t="inlineStr">
         <is>
-          <t>High-volume prospectors</t>
+          <t>SDRs needing quick contact data</t>
         </is>
       </c>
       <c r="K210" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L210" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M210" s="5" t="n">
         <v>6</v>
       </c>
       <c r="N210" s="5" t="n">
-        <v>5</v>
+        <v>5.7</v>
       </c>
       <c r="O210" s="5" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="211" ht="58" customHeight="1">
       <c r="A211" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=instantly.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=seamless.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B211" s="6" t="inlineStr">
         <is>
-          <t>Instantly</t>
+          <t>Seamless.AI</t>
         </is>
       </c>
       <c r="C211" s="7" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Freemium</t>
         </is>
       </c>
       <c r="D211" s="8" t="inlineStr">
         <is>
-          <t>instantly.ai</t>
+          <t>seamless.ai</t>
         </is>
       </c>
       <c r="E211" s="7" t="inlineStr">
         <is>
-          <t>Cold email at scale: warmup, inbox rotation, deliverability, AI writing</t>
+          <t>Real-time AI search engine for B2B contact information</t>
         </is>
       </c>
       <c r="F211" s="7" t="inlineStr">
         <is>
-          <t>From $37/mo</t>
+          <t>Free credits; from ~$147/mo</t>
         </is>
       </c>
       <c r="G211" s="7" t="inlineStr">
@@ -13604,43 +13604,43 @@
       </c>
       <c r="H211" s="7" t="inlineStr">
         <is>
-          <t>Best-known deliverability stack; unlimited sending accounts</t>
+          <t>Real-time verification; high volumes</t>
         </is>
       </c>
       <c r="I211" s="7" t="inlineStr">
         <is>
-          <t>Cold-email compliance is on you</t>
+          <t>Data-accuracy complaints; pushy sales motion</t>
         </is>
       </c>
       <c r="J211" s="7" t="inlineStr">
         <is>
-          <t>Agencies and outbound startups</t>
+          <t>High-volume prospectors</t>
         </is>
       </c>
       <c r="K211" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L211" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="L211" s="5" t="n">
-        <v>7</v>
-      </c>
       <c r="M211" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N211" s="5" t="n">
-        <v>6.3</v>
+        <v>5</v>
       </c>
       <c r="O211" s="5" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
     </row>
     <row r="212" ht="58" customHeight="1">
       <c r="A212" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=smartlead.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=instantly.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B212" s="6" t="inlineStr">
         <is>
-          <t>Smartlead</t>
+          <t>Instantly</t>
         </is>
       </c>
       <c r="C212" s="7" t="inlineStr">
@@ -13650,17 +13650,17 @@
       </c>
       <c r="D212" s="8" t="inlineStr">
         <is>
-          <t>smartlead.ai</t>
+          <t>instantly.ai</t>
         </is>
       </c>
       <c r="E212" s="7" t="inlineStr">
         <is>
-          <t>Cold email infrastructure with unlimited mailboxes and AI warmup</t>
+          <t>Cold email at scale: warmup, inbox rotation, deliverability, AI writing</t>
         </is>
       </c>
       <c r="F212" s="7" t="inlineStr">
         <is>
-          <t>From $39/mo</t>
+          <t>From $37/mo</t>
         </is>
       </c>
       <c r="G212" s="7" t="inlineStr">
@@ -13670,17 +13670,17 @@
       </c>
       <c r="H212" s="7" t="inlineStr">
         <is>
-          <t>Unlimited mailboxes; API-first</t>
+          <t>Best-known deliverability stack; unlimited sending accounts</t>
         </is>
       </c>
       <c r="I212" s="7" t="inlineStr">
         <is>
-          <t>UI rough edges</t>
+          <t>Cold-email compliance is on you</t>
         </is>
       </c>
       <c r="J212" s="7" t="inlineStr">
         <is>
-          <t>Outbound agencies</t>
+          <t>Agencies and outbound startups</t>
         </is>
       </c>
       <c r="K212" s="5" t="n">
@@ -13696,17 +13696,17 @@
         <v>6.3</v>
       </c>
       <c r="O212" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="213" ht="58" customHeight="1">
       <c r="A213" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=lemlist.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=smartlead.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B213" s="6" t="inlineStr">
         <is>
-          <t>lemlist</t>
+          <t>Smartlead</t>
         </is>
       </c>
       <c r="C213" s="7" t="inlineStr">
@@ -13716,17 +13716,17 @@
       </c>
       <c r="D213" s="8" t="inlineStr">
         <is>
-          <t>lemlist.com</t>
+          <t>smartlead.ai</t>
         </is>
       </c>
       <c r="E213" s="7" t="inlineStr">
         <is>
-          <t>Multichannel outreach (email/LinkedIn/calls) with AI personalisation</t>
+          <t>Cold email infrastructure with unlimited mailboxes and AI warmup</t>
         </is>
       </c>
       <c r="F213" s="7" t="inlineStr">
         <is>
-          <t>From $39/user/mo</t>
+          <t>From $39/mo</t>
         </is>
       </c>
       <c r="G213" s="7" t="inlineStr">
@@ -13736,43 +13736,43 @@
       </c>
       <c r="H213" s="7" t="inlineStr">
         <is>
-          <t>Strong personalisation (images, dynamic content)</t>
+          <t>Unlimited mailboxes; API-first</t>
         </is>
       </c>
       <c r="I213" s="7" t="inlineStr">
         <is>
-          <t>Per-seat costs add up</t>
+          <t>UI rough edges</t>
         </is>
       </c>
       <c r="J213" s="7" t="inlineStr">
         <is>
-          <t>SDRs doing personalised sequences</t>
+          <t>Outbound agencies</t>
         </is>
       </c>
       <c r="K213" s="5" t="n">
         <v>5</v>
       </c>
       <c r="L213" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M213" s="5" t="n">
         <v>7</v>
       </c>
       <c r="N213" s="5" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="O213" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="214" ht="58" customHeight="1">
       <c r="A214" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=reply.io&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=lemlist.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B214" s="6" t="inlineStr">
         <is>
-          <t>Reply.io</t>
+          <t>lemlist</t>
         </is>
       </c>
       <c r="C214" s="7" t="inlineStr">
@@ -13782,17 +13782,17 @@
       </c>
       <c r="D214" s="8" t="inlineStr">
         <is>
-          <t>reply.io</t>
+          <t>lemlist.com</t>
         </is>
       </c>
       <c r="E214" s="7" t="inlineStr">
         <is>
-          <t>AI SDR agents plus multichannel sales sequences</t>
+          <t>Multichannel outreach (email/LinkedIn/calls) with AI personalisation</t>
         </is>
       </c>
       <c r="F214" s="7" t="inlineStr">
         <is>
-          <t>From $59/user/mo; AI SDR from ~$259/mo</t>
+          <t>From $39/user/mo</t>
         </is>
       </c>
       <c r="G214" s="7" t="inlineStr">
@@ -13802,17 +13802,17 @@
       </c>
       <c r="H214" s="7" t="inlineStr">
         <is>
-          <t>Mature sequencer with AI-agent option</t>
+          <t>Strong personalisation (images, dynamic content)</t>
         </is>
       </c>
       <c r="I214" s="7" t="inlineStr">
         <is>
-          <t>AI-agent quality varies</t>
+          <t>Per-seat costs add up</t>
         </is>
       </c>
       <c r="J214" s="7" t="inlineStr">
         <is>
-          <t>Lean teams automating outreach</t>
+          <t>SDRs doing personalised sequences</t>
         </is>
       </c>
       <c r="K214" s="5" t="n">
@@ -13828,17 +13828,17 @@
         <v>6</v>
       </c>
       <c r="O214" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="215" ht="58" customHeight="1">
       <c r="A215" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=qualified.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=reply.io&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B215" s="6" t="inlineStr">
         <is>
-          <t>Qualified</t>
+          <t>Reply.io</t>
         </is>
       </c>
       <c r="C215" s="7" t="inlineStr">
@@ -13848,17 +13848,17 @@
       </c>
       <c r="D215" s="8" t="inlineStr">
         <is>
-          <t>qualified.com</t>
+          <t>reply.io</t>
         </is>
       </c>
       <c r="E215" s="7" t="inlineStr">
         <is>
-          <t>AI SDR 'Piper' converts website visitors into pipeline (Salesforce-native)</t>
+          <t>AI SDR agents plus multichannel sales sequences</t>
         </is>
       </c>
       <c r="F215" s="7" t="inlineStr">
         <is>
-          <t>From ~$3,500/mo</t>
+          <t>From $59/user/mo; AI SDR from ~$259/mo</t>
         </is>
       </c>
       <c r="G215" s="7" t="inlineStr">
@@ -13868,43 +13868,43 @@
       </c>
       <c r="H215" s="7" t="inlineStr">
         <is>
-          <t>Best-in-class inbound conversion for Salesforce shops</t>
+          <t>Mature sequencer with AI-agent option</t>
         </is>
       </c>
       <c r="I215" s="7" t="inlineStr">
         <is>
-          <t>Enterprise pricing; Salesforce required</t>
+          <t>AI-agent quality varies</t>
         </is>
       </c>
       <c r="J215" s="7" t="inlineStr">
         <is>
-          <t>Enterprise demand-gen teams</t>
+          <t>Lean teams automating outreach</t>
         </is>
       </c>
       <c r="K215" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L215" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M215" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N215" s="5" t="n">
-        <v>5.7</v>
+        <v>6</v>
       </c>
       <c r="O215" s="5" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="216" ht="58" customHeight="1">
       <c r="A216" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=11x.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=qualified.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B216" s="6" t="inlineStr">
         <is>
-          <t>11x</t>
+          <t>Qualified</t>
         </is>
       </c>
       <c r="C216" s="7" t="inlineStr">
@@ -13914,17 +13914,17 @@
       </c>
       <c r="D216" s="8" t="inlineStr">
         <is>
-          <t>11x.ai</t>
+          <t>qualified.com</t>
         </is>
       </c>
       <c r="E216" s="7" t="inlineStr">
         <is>
-          <t>Autonomous 'digital worker' AI SDRs (Alice) running outbound end-to-end</t>
+          <t>AI SDR 'Piper' converts website visitors into pipeline (Salesforce-native)</t>
         </is>
       </c>
       <c r="F216" s="7" t="inlineStr">
         <is>
-          <t>Custom (thousands/mo)</t>
+          <t>From ~$3,500/mo</t>
         </is>
       </c>
       <c r="G216" s="7" t="inlineStr">
@@ -13934,43 +13934,43 @@
       </c>
       <c r="H216" s="7" t="inlineStr">
         <is>
-          <t>Fully autonomous outbound experiments</t>
+          <t>Best-in-class inbound conversion for Salesforce shops</t>
         </is>
       </c>
       <c r="I216" s="7" t="inlineStr">
         <is>
-          <t>Mixed quality reports; hype-heavy category</t>
+          <t>Enterprise pricing; Salesforce required</t>
         </is>
       </c>
       <c r="J216" s="7" t="inlineStr">
         <is>
-          <t>Teams experimenting with AI SDRs</t>
+          <t>Enterprise demand-gen teams</t>
         </is>
       </c>
       <c r="K216" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L216" s="5" t="n">
         <v>3</v>
       </c>
       <c r="M216" s="5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N216" s="5" t="n">
-        <v>4.3</v>
+        <v>5.7</v>
       </c>
       <c r="O216" s="5" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="217" ht="58" customHeight="1">
       <c r="A217" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=artisan.co&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=11x.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B217" s="6" t="inlineStr">
         <is>
-          <t>Artisan</t>
+          <t>11x</t>
         </is>
       </c>
       <c r="C217" s="7" t="inlineStr">
@@ -13980,17 +13980,17 @@
       </c>
       <c r="D217" s="8" t="inlineStr">
         <is>
-          <t>artisan.co</t>
+          <t>11x.ai</t>
         </is>
       </c>
       <c r="E217" s="7" t="inlineStr">
         <is>
-          <t>AI BDR 'Ava': finds leads, researches, writes and sends outbound</t>
+          <t>Autonomous 'digital worker' AI SDRs (Alice) running outbound end-to-end</t>
         </is>
       </c>
       <c r="F217" s="7" t="inlineStr">
         <is>
-          <t>Custom (from ~$2k/mo)</t>
+          <t>Custom (thousands/mo)</t>
         </is>
       </c>
       <c r="G217" s="7" t="inlineStr">
@@ -14000,17 +14000,17 @@
       </c>
       <c r="H217" s="7" t="inlineStr">
         <is>
-          <t>Consolidates data + email infra + AI in one</t>
+          <t>Fully autonomous outbound experiments</t>
         </is>
       </c>
       <c r="I217" s="7" t="inlineStr">
         <is>
-          <t>Young product; needs supervision</t>
+          <t>Mixed quality reports; hype-heavy category</t>
         </is>
       </c>
       <c r="J217" s="7" t="inlineStr">
         <is>
-          <t>Startups without SDR headcount</t>
+          <t>Teams experimenting with AI SDRs</t>
         </is>
       </c>
       <c r="K217" s="5" t="n">
@@ -14026,17 +14026,17 @@
         <v>4.3</v>
       </c>
       <c r="O217" s="5" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="218" ht="58" customHeight="1">
       <c r="A218" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=nooks.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=artisan.co&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B218" s="6" t="inlineStr">
         <is>
-          <t>Nooks</t>
+          <t>Artisan</t>
         </is>
       </c>
       <c r="C218" s="7" t="inlineStr">
@@ -14046,17 +14046,17 @@
       </c>
       <c r="D218" s="8" t="inlineStr">
         <is>
-          <t>nooks.ai</t>
+          <t>artisan.co</t>
         </is>
       </c>
       <c r="E218" s="7" t="inlineStr">
         <is>
-          <t>AI parallel dialer, virtual salesfloor and call coaching</t>
+          <t>AI BDR 'Ava': finds leads, researches, writes and sends outbound</t>
         </is>
       </c>
       <c r="F218" s="7" t="inlineStr">
         <is>
-          <t>Custom (~$200/user/mo)</t>
+          <t>Custom (from ~$2k/mo)</t>
         </is>
       </c>
       <c r="G218" s="7" t="inlineStr">
@@ -14066,63 +14066,63 @@
       </c>
       <c r="H218" s="7" t="inlineStr">
         <is>
-          <t>3-5x connect rates for calling teams</t>
+          <t>Consolidates data + email infra + AI in one</t>
         </is>
       </c>
       <c r="I218" s="7" t="inlineStr">
         <is>
-          <t>Dialer-centric; custom pricing</t>
+          <t>Young product; needs supervision</t>
         </is>
       </c>
       <c r="J218" s="7" t="inlineStr">
         <is>
-          <t>Cold-calling SDR teams</t>
+          <t>Startups without SDR headcount</t>
         </is>
       </c>
       <c r="K218" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L218" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M218" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N218" s="5" t="n">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
       <c r="O218" s="5" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
     </row>
     <row r="219" ht="58" customHeight="1">
       <c r="A219" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=warmly.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=nooks.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B219" s="6" t="inlineStr">
         <is>
-          <t>Warmly</t>
+          <t>Nooks</t>
         </is>
       </c>
       <c r="C219" s="7" t="inlineStr">
         <is>
-          <t>Freemium</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="D219" s="8" t="inlineStr">
         <is>
-          <t>warmly.ai</t>
+          <t>nooks.ai</t>
         </is>
       </c>
       <c r="E219" s="7" t="inlineStr">
         <is>
-          <t>De-anonymises website visitors and orchestrates AI outreach to them</t>
+          <t>AI parallel dialer, virtual salesfloor and call coaching</t>
         </is>
       </c>
       <c r="F219" s="7" t="inlineStr">
         <is>
-          <t>Free; from ~$700/mo</t>
+          <t>Custom (~$200/user/mo)</t>
         </is>
       </c>
       <c r="G219" s="7" t="inlineStr">
@@ -14132,43 +14132,43 @@
       </c>
       <c r="H219" s="7" t="inlineStr">
         <is>
-          <t>Good intent signals for the price</t>
+          <t>3-5x connect rates for calling teams</t>
         </is>
       </c>
       <c r="I219" s="7" t="inlineStr">
         <is>
-          <t>Pricing jumps sharply after free tier</t>
+          <t>Dialer-centric; custom pricing</t>
         </is>
       </c>
       <c r="J219" s="7" t="inlineStr">
         <is>
-          <t>SMB pipeline teams</t>
+          <t>Cold-calling SDR teams</t>
         </is>
       </c>
       <c r="K219" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L219" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="L219" s="5" t="n">
-        <v>5</v>
-      </c>
       <c r="M219" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N219" s="5" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="O219" s="5" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="220" ht="58" customHeight="1">
       <c r="A220" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=crystalknows.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=warmly.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B220" s="6" t="inlineStr">
         <is>
-          <t>Crystal</t>
+          <t>Warmly</t>
         </is>
       </c>
       <c r="C220" s="7" t="inlineStr">
@@ -14178,17 +14178,17 @@
       </c>
       <c r="D220" s="8" t="inlineStr">
         <is>
-          <t>crystalknows.com</t>
+          <t>warmly.ai</t>
         </is>
       </c>
       <c r="E220" s="7" t="inlineStr">
         <is>
-          <t>DISC personality profiles for prospects to tailor messaging</t>
+          <t>De-anonymises website visitors and orchestrates AI outreach to them</t>
         </is>
       </c>
       <c r="F220" s="7" t="inlineStr">
         <is>
-          <t>Free; from $49/mo</t>
+          <t>Free; from ~$700/mo</t>
         </is>
       </c>
       <c r="G220" s="7" t="inlineStr">
@@ -14198,17 +14198,17 @@
       </c>
       <c r="H220" s="7" t="inlineStr">
         <is>
-          <t>Unique personality-based angle</t>
+          <t>Good intent signals for the price</t>
         </is>
       </c>
       <c r="I220" s="7" t="inlineStr">
         <is>
-          <t>Profile accuracy varies</t>
+          <t>Pricing jumps sharply after free tier</t>
         </is>
       </c>
       <c r="J220" s="7" t="inlineStr">
         <is>
-          <t>Relationship-driven sellers</t>
+          <t>SMB pipeline teams</t>
         </is>
       </c>
       <c r="K220" s="5" t="n">
@@ -14224,37 +14224,37 @@
         <v>5</v>
       </c>
       <c r="O220" s="5" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="221" ht="58" customHeight="1">
       <c r="A221" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=regie.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=crystalknows.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B221" s="6" t="inlineStr">
         <is>
-          <t>Regie.ai</t>
+          <t>Crystal</t>
         </is>
       </c>
       <c r="C221" s="7" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Freemium</t>
         </is>
       </c>
       <c r="D221" s="8" t="inlineStr">
         <is>
-          <t>regie.ai</t>
+          <t>crystalknows.com</t>
         </is>
       </c>
       <c r="E221" s="7" t="inlineStr">
         <is>
-          <t>Generative AI platform for sales prospecting content and sequencing</t>
+          <t>DISC personality profiles for prospects to tailor messaging</t>
         </is>
       </c>
       <c r="F221" s="7" t="inlineStr">
         <is>
-          <t>Custom pricing</t>
+          <t>Free; from $49/mo</t>
         </is>
       </c>
       <c r="G221" s="7" t="inlineStr">
@@ -14264,43 +14264,43 @@
       </c>
       <c r="H221" s="7" t="inlineStr">
         <is>
-          <t>Brand-controlled AI sales content at scale</t>
+          <t>Unique personality-based angle</t>
         </is>
       </c>
       <c r="I221" s="7" t="inlineStr">
         <is>
-          <t>Opaque pricing</t>
+          <t>Profile accuracy varies</t>
         </is>
       </c>
       <c r="J221" s="7" t="inlineStr">
         <is>
-          <t>Enterprise SDR organisations</t>
+          <t>Relationship-driven sellers</t>
         </is>
       </c>
       <c r="K221" s="5" t="n">
         <v>4</v>
       </c>
       <c r="L221" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M221" s="5" t="n">
         <v>6</v>
       </c>
       <c r="N221" s="5" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="O221" s="5" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="222" ht="58" customHeight="1">
       <c r="A222" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=salesape.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=regie.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B222" s="6" t="inlineStr">
         <is>
-          <t>SalesAPE.ai</t>
+          <t>Regie.ai</t>
         </is>
       </c>
       <c r="C222" s="7" t="inlineStr">
@@ -14310,17 +14310,17 @@
       </c>
       <c r="D222" s="8" t="inlineStr">
         <is>
-          <t>salesape.ai</t>
+          <t>regie.ai</t>
         </is>
       </c>
       <c r="E222" s="7" t="inlineStr">
         <is>
-          <t>AI inbound sales agent: qualifies leads via chat/SMS/WhatsApp/email and books meetings 24/7</t>
+          <t>Generative AI platform for sales prospecting content and sequencing</t>
         </is>
       </c>
       <c r="F222" s="7" t="inlineStr">
         <is>
-          <t>~$999/mo + ~$3k setup (quote-based)</t>
+          <t>Custom pricing</t>
         </is>
       </c>
       <c r="G222" s="7" t="inlineStr">
@@ -14330,17 +14330,17 @@
       </c>
       <c r="H222" s="7" t="inlineStr">
         <is>
-          <t>Responds to inbound leads in seconds across channels</t>
+          <t>Brand-controlled AI sales content at scale</t>
         </is>
       </c>
       <c r="I222" s="7" t="inlineStr">
         <is>
-          <t>Quote-only pricing; setup fee</t>
+          <t>Opaque pricing</t>
         </is>
       </c>
       <c r="J222" s="7" t="inlineStr">
         <is>
-          <t>SMBs losing inbound leads to slow follow-up</t>
+          <t>Enterprise SDR organisations</t>
         </is>
       </c>
       <c r="K222" s="5" t="n">
@@ -14350,23 +14350,23 @@
         <v>4</v>
       </c>
       <c r="M222" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N222" s="5" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="O222" s="5" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="223" ht="58" customHeight="1">
       <c r="A223" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=altahq.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=salesape.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B223" s="6" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>SalesAPE.ai</t>
         </is>
       </c>
       <c r="C223" s="7" t="inlineStr">
@@ -14376,17 +14376,17 @@
       </c>
       <c r="D223" s="8" t="inlineStr">
         <is>
-          <t>altahq.com</t>
+          <t>salesape.ai</t>
         </is>
       </c>
       <c r="E223" s="7" t="inlineStr">
         <is>
-          <t>AI GTM agent team (Katie SDR, Alex calling, Luna analytics) on one shared data layer</t>
+          <t>AI inbound sales agent: qualifies leads via chat/SMS/WhatsApp/email and books meetings 24/7</t>
         </is>
       </c>
       <c r="F223" s="7" t="inlineStr">
         <is>
-          <t>Custom platform fee</t>
+          <t>~$999/mo + ~$3k setup (quote-based)</t>
         </is>
       </c>
       <c r="G223" s="7" t="inlineStr">
@@ -14396,43 +14396,43 @@
       </c>
       <c r="H223" s="7" t="inlineStr">
         <is>
-          <t>Full agent team incl. voice; Salesforce app; used by Snowflake/Deel</t>
+          <t>Responds to inbound leads in seconds across channels</t>
         </is>
       </c>
       <c r="I223" s="7" t="inlineStr">
         <is>
-          <t>Custom pricing; newer vendor</t>
+          <t>Quote-only pricing; setup fee</t>
         </is>
       </c>
       <c r="J223" s="7" t="inlineStr">
         <is>
-          <t>B2B teams automating top-of-funnel</t>
+          <t>SMBs losing inbound leads to slow follow-up</t>
         </is>
       </c>
       <c r="K223" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L223" s="5" t="n">
         <v>4</v>
       </c>
       <c r="M223" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N223" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O223" s="5" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="224" ht="58" customHeight="1">
       <c r="A224" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=salescloser.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=altahq.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B224" s="6" t="inlineStr">
         <is>
-          <t>SalesCloser AI</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="C224" s="7" t="inlineStr">
@@ -14442,17 +14442,17 @@
       </c>
       <c r="D224" s="8" t="inlineStr">
         <is>
-          <t>salescloser.ai</t>
+          <t>altahq.com</t>
         </is>
       </c>
       <c r="E224" s="7" t="inlineStr">
         <is>
-          <t>AI sales agent that runs discovery and demo calls over phone/Zoom in 32+ languages, 24/7</t>
+          <t>AI GTM agent team (Katie SDR, Alex calling, Luna analytics) on one shared data layer</t>
         </is>
       </c>
       <c r="F224" s="7" t="inlineStr">
         <is>
-          <t>From $1,000/mo; Enterprise $2,500/mo</t>
+          <t>Custom platform fee</t>
         </is>
       </c>
       <c r="G224" s="7" t="inlineStr">
@@ -14462,43 +14462,43 @@
       </c>
       <c r="H224" s="7" t="inlineStr">
         <is>
-          <t>Flat-rate pricing; screen-share demos; multilingual</t>
+          <t>Full agent team incl. voice; Salesforce app; used by Snowflake/Deel</t>
         </is>
       </c>
       <c r="I224" s="7" t="inlineStr">
         <is>
-          <t>Trusting AI to run sales calls suits simple products best</t>
+          <t>Custom pricing; newer vendor</t>
         </is>
       </c>
       <c r="J224" s="7" t="inlineStr">
         <is>
-          <t>SaaS with high-volume, simple demos</t>
+          <t>B2B teams automating top-of-funnel</t>
         </is>
       </c>
       <c r="K224" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L224" s="5" t="n">
         <v>4</v>
       </c>
       <c r="M224" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N224" s="5" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
       <c r="O224" s="5" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="225" ht="58" customHeight="1">
       <c r="A225" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=aisdr.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=salescloser.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B225" s="6" t="inlineStr">
         <is>
-          <t>AiSDR</t>
+          <t>SalesCloser AI</t>
         </is>
       </c>
       <c r="C225" s="7" t="inlineStr">
@@ -14508,17 +14508,17 @@
       </c>
       <c r="D225" s="8" t="inlineStr">
         <is>
-          <t>aisdr.com</t>
+          <t>salescloser.ai</t>
         </is>
       </c>
       <c r="E225" s="7" t="inlineStr">
         <is>
-          <t>AI SDR for email + LinkedIn outreach with HubSpot/Salesforce integration</t>
+          <t>AI sales agent that runs discovery and demo calls over phone/Zoom in 32+ languages, 24/7</t>
         </is>
       </c>
       <c r="F225" s="7" t="inlineStr">
         <is>
-          <t>From $900/mo (1,200 messages)</t>
+          <t>From $1,000/mo; Enterprise $2,500/mo</t>
         </is>
       </c>
       <c r="G225" s="7" t="inlineStr">
@@ -14528,17 +14528,17 @@
       </c>
       <c r="H225" s="7" t="inlineStr">
         <is>
-          <t>Transparent pricing; solid CRM integrations</t>
+          <t>Flat-rate pricing; screen-share demos; multilingual</t>
         </is>
       </c>
       <c r="I225" s="7" t="inlineStr">
         <is>
-          <t>Feature set reflects the price point</t>
+          <t>Trusting AI to run sales calls suits simple products best</t>
         </is>
       </c>
       <c r="J225" s="7" t="inlineStr">
         <is>
-          <t>Teams testing AI SDRs without enterprise contracts</t>
+          <t>SaaS with high-volume, simple demos</t>
         </is>
       </c>
       <c r="K225" s="5" t="n">
@@ -14554,17 +14554,17 @@
         <v>5.3</v>
       </c>
       <c r="O225" s="5" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="226" ht="58" customHeight="1">
       <c r="A226" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=salesforge.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=aisdr.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B226" s="6" t="inlineStr">
         <is>
-          <t>Salesforge</t>
+          <t>AiSDR</t>
         </is>
       </c>
       <c r="C226" s="7" t="inlineStr">
@@ -14574,17 +14574,17 @@
       </c>
       <c r="D226" s="8" t="inlineStr">
         <is>
-          <t>salesforge.ai</t>
+          <t>aisdr.com</t>
         </is>
       </c>
       <c r="E226" s="7" t="inlineStr">
         <is>
-          <t>Cold email platform with 'Agent Frank', an AI SDR in co-pilot or autopilot mode</t>
+          <t>AI SDR for email + LinkedIn outreach with HubSpot/Salesforce integration</t>
         </is>
       </c>
       <c r="F226" s="7" t="inlineStr">
         <is>
-          <t>From $40/mo; Agent Frank from $416/mo</t>
+          <t>From $900/mo (1,200 messages)</t>
         </is>
       </c>
       <c r="G226" s="7" t="inlineStr">
@@ -14594,43 +14594,43 @@
       </c>
       <c r="H226" s="7" t="inlineStr">
         <is>
-          <t>Co-pilot mode keeps humans in the loop; good deliverability</t>
+          <t>Transparent pricing; solid CRM integrations</t>
         </is>
       </c>
       <c r="I226" s="7" t="inlineStr">
         <is>
-          <t>Email-focused</t>
+          <t>Feature set reflects the price point</t>
         </is>
       </c>
       <c r="J226" s="7" t="inlineStr">
         <is>
-          <t>Lean outbound teams</t>
+          <t>Teams testing AI SDRs without enterprise contracts</t>
         </is>
       </c>
       <c r="K226" s="5" t="n">
         <v>5</v>
       </c>
       <c r="L226" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M226" s="5" t="n">
         <v>7</v>
       </c>
       <c r="N226" s="5" t="n">
-        <v>6</v>
+        <v>5.3</v>
       </c>
       <c r="O226" s="5" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="227" ht="58" customHeight="1">
       <c r="A227" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=amplemarket.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=salesforge.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B227" s="6" t="inlineStr">
         <is>
-          <t>Amplemarket</t>
+          <t>Salesforge</t>
         </is>
       </c>
       <c r="C227" s="7" t="inlineStr">
@@ -14640,17 +14640,17 @@
       </c>
       <c r="D227" s="8" t="inlineStr">
         <is>
-          <t>amplemarket.com</t>
+          <t>salesforge.ai</t>
         </is>
       </c>
       <c r="E227" s="7" t="inlineStr">
         <is>
-          <t>AI sales platform with 'Duo' copilot: B2B data, sequencing and AI in one</t>
+          <t>Cold email platform with 'Agent Frank', an AI SDR in co-pilot or autopilot mode</t>
         </is>
       </c>
       <c r="F227" s="7" t="inlineStr">
         <is>
-          <t>~$3,200/user/yr (annual contracts)</t>
+          <t>From $40/mo; Agent Frank from $416/mo</t>
         </is>
       </c>
       <c r="G227" s="7" t="inlineStr">
@@ -14660,175 +14660,175 @@
       </c>
       <c r="H227" s="7" t="inlineStr">
         <is>
-          <t>Human+AI Duo approach; all-in-one data + outreach</t>
+          <t>Co-pilot mode keeps humans in the loop; good deliverability</t>
         </is>
       </c>
       <c r="I227" s="7" t="inlineStr">
         <is>
-          <t>Annual commitment; pricier per seat</t>
+          <t>Email-focused</t>
         </is>
       </c>
       <c r="J227" s="7" t="inlineStr">
         <is>
-          <t>Mid-market outbound teams</t>
+          <t>Lean outbound teams</t>
         </is>
       </c>
       <c r="K227" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L227" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M227" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N227" s="5" t="n">
         <v>6</v>
       </c>
       <c r="O227" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="228" ht="58" customHeight="1">
       <c r="A228" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=relevanceai.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=amplemarket.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B228" s="6" t="inlineStr">
         <is>
-          <t>Relevance AI</t>
+          <t>Amplemarket</t>
         </is>
       </c>
       <c r="C228" s="7" t="inlineStr">
         <is>
-          <t>Freemium</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="D228" s="8" t="inlineStr">
         <is>
-          <t>relevanceai.com</t>
+          <t>amplemarket.com</t>
         </is>
       </c>
       <c r="E228" s="7" t="inlineStr">
         <is>
-          <t>No-code AI workforce builder: custom sales agents (incl. Bosh AI BDR) and workflows</t>
+          <t>AI sales platform with 'Duo' copilot: B2B data, sequencing and AI in one</t>
         </is>
       </c>
       <c r="F228" s="7" t="inlineStr">
         <is>
-          <t>Free tier; from ~$19/mo + usage</t>
+          <t>~$3,200/user/yr (annual contracts)</t>
         </is>
       </c>
       <c r="G228" s="7" t="inlineStr">
         <is>
-          <t>Yes — Claude selectable as the agent model</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H228" s="7" t="inlineStr">
         <is>
-          <t>Build exactly the agent you want without code</t>
+          <t>Human+AI Duo approach; all-in-one data + outreach</t>
         </is>
       </c>
       <c r="I228" s="7" t="inlineStr">
         <is>
-          <t>More setup than turnkey AI SDRs</t>
+          <t>Annual commitment; pricier per seat</t>
         </is>
       </c>
       <c r="J228" s="7" t="inlineStr">
         <is>
-          <t>RevOps teams building custom agents</t>
+          <t>Mid-market outbound teams</t>
         </is>
       </c>
       <c r="K228" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L228" s="5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M228" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N228" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O228" s="5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="229" ht="58" customHeight="1">
       <c r="A229" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=unifygtm.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=relevanceai.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B229" s="6" t="inlineStr">
         <is>
-          <t>Unify</t>
+          <t>Relevance AI</t>
         </is>
       </c>
       <c r="C229" s="7" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Freemium</t>
         </is>
       </c>
       <c r="D229" s="8" t="inlineStr">
         <is>
-          <t>unifygtm.com</t>
+          <t>relevanceai.com</t>
         </is>
       </c>
       <c r="E229" s="7" t="inlineStr">
         <is>
-          <t>Warm outbound: buying signals, website intent and AI-personalised sequences</t>
+          <t>No-code AI workforce builder: custom sales agents (incl. Bosh AI BDR) and workflows</t>
         </is>
       </c>
       <c r="F229" s="7" t="inlineStr">
         <is>
-          <t>From ~$700/mo (custom)</t>
+          <t>Free tier; from ~$19/mo + usage</t>
         </is>
       </c>
       <c r="G229" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes — Claude selectable as the agent model</t>
         </is>
       </c>
       <c r="H229" s="7" t="inlineStr">
         <is>
-          <t>Signal-based outbound beats cold lists</t>
+          <t>Build exactly the agent you want without code</t>
         </is>
       </c>
       <c r="I229" s="7" t="inlineStr">
         <is>
-          <t>Price; needs traffic/signals to shine</t>
+          <t>More setup than turnkey AI SDRs</t>
         </is>
       </c>
       <c r="J229" s="7" t="inlineStr">
         <is>
-          <t>PLG and mid-market growth teams</t>
+          <t>RevOps teams building custom agents</t>
         </is>
       </c>
       <c r="K229" s="5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L229" s="5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M229" s="5" t="n">
         <v>7</v>
       </c>
       <c r="N229" s="5" t="n">
-        <v>5.3</v>
+        <v>7</v>
       </c>
       <c r="O229" s="5" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
     </row>
     <row r="230" ht="58" customHeight="1">
       <c r="A230" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=commonroom.io&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=unifygtm.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B230" s="6" t="inlineStr">
         <is>
-          <t>Common Room</t>
+          <t>Unify</t>
         </is>
       </c>
       <c r="C230" s="7" t="inlineStr">
@@ -14838,17 +14838,17 @@
       </c>
       <c r="D230" s="8" t="inlineStr">
         <is>
-          <t>commonroom.io</t>
+          <t>unifygtm.com</t>
         </is>
       </c>
       <c r="E230" s="7" t="inlineStr">
         <is>
-          <t>Customer intelligence: aggregates community, product and social signals for GTM (RoomieAI)</t>
+          <t>Warm outbound: buying signals, website intent and AI-personalised sequences</t>
         </is>
       </c>
       <c r="F230" s="7" t="inlineStr">
         <is>
-          <t>From ~$999/mo</t>
+          <t>From ~$700/mo (custom)</t>
         </is>
       </c>
       <c r="G230" s="7" t="inlineStr">
@@ -14858,248 +14858,248 @@
       </c>
       <c r="H230" s="7" t="inlineStr">
         <is>
-          <t>Unmatched signal coverage (30+ channels)</t>
+          <t>Signal-based outbound beats cold lists</t>
         </is>
       </c>
       <c r="I230" s="7" t="inlineStr">
         <is>
-          <t>Cost; needs dedicated ops attention</t>
+          <t>Price; needs traffic/signals to shine</t>
         </is>
       </c>
       <c r="J230" s="7" t="inlineStr">
         <is>
-          <t>DevTool and PLG companies</t>
+          <t>PLG and mid-market growth teams</t>
         </is>
       </c>
       <c r="K230" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L230" s="5" t="n">
         <v>4</v>
       </c>
       <c r="M230" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N230" s="5" t="n">
-        <v>6</v>
+        <v>5.3</v>
       </c>
       <c r="O230" s="5" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="231" ht="58" customHeight="1">
       <c r="A231" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=commonroom.io&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B231" s="6" t="inlineStr">
+        <is>
+          <t>Common Room</t>
+        </is>
+      </c>
+      <c r="C231" s="7" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D231" s="8" t="inlineStr">
+        <is>
+          <t>commonroom.io</t>
+        </is>
+      </c>
+      <c r="E231" s="7" t="inlineStr">
+        <is>
+          <t>Customer intelligence: aggregates community, product and social signals for GTM (RoomieAI)</t>
+        </is>
+      </c>
+      <c r="F231" s="7" t="inlineStr">
+        <is>
+          <t>From ~$999/mo</t>
+        </is>
+      </c>
+      <c r="G231" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H231" s="7" t="inlineStr">
+        <is>
+          <t>Unmatched signal coverage (30+ channels)</t>
+        </is>
+      </c>
+      <c r="I231" s="7" t="inlineStr">
+        <is>
+          <t>Cost; needs dedicated ops attention</t>
+        </is>
+      </c>
+      <c r="J231" s="7" t="inlineStr">
+        <is>
+          <t>DevTool and PLG companies</t>
+        </is>
+      </c>
+      <c r="K231" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L231" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M231" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="N231" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="O231" s="5" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="232" ht="58" customHeight="1">
+      <c r="A232" s="5">
         <f>IMAGE("https://www.google.com/s2/favicons?domain=humantic.ai&amp;sz=64")</f>
         <v/>
       </c>
-      <c r="B231" s="6" t="inlineStr">
+      <c r="B232" s="6" t="inlineStr">
         <is>
           <t>Humantic AI</t>
         </is>
       </c>
-      <c r="C231" s="7" t="inlineStr">
+      <c r="C232" s="7" t="inlineStr">
         <is>
           <t>Freemium</t>
         </is>
       </c>
-      <c r="D231" s="8" t="inlineStr">
+      <c r="D232" s="8" t="inlineStr">
         <is>
           <t>humantic.ai</t>
         </is>
       </c>
-      <c r="E231" s="7" t="inlineStr">
+      <c r="E232" s="7" t="inlineStr">
         <is>
           <t>Buyer personality intelligence (DISC) for personalised selling in LinkedIn/CRM</t>
         </is>
       </c>
-      <c r="F231" s="7" t="inlineStr">
+      <c r="F232" s="7" t="inlineStr">
         <is>
           <t>Free trial; from ~$30/mo</t>
         </is>
       </c>
-      <c r="G231" s="7" t="inlineStr">
+      <c r="G232" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H231" s="7" t="inlineStr">
+      <c r="H232" s="7" t="inlineStr">
         <is>
           <t>Personality insights where you work</t>
         </is>
       </c>
-      <c r="I231" s="7" t="inlineStr">
+      <c r="I232" s="7" t="inlineStr">
         <is>
           <t>Accuracy debatable; niche</t>
         </is>
       </c>
-      <c r="J231" s="7" t="inlineStr">
+      <c r="J232" s="7" t="inlineStr">
         <is>
           <t>Enterprise AEs personalising outreach</t>
         </is>
       </c>
-      <c r="K231" s="5" t="n">
+      <c r="K232" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="L231" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="M231" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N231" s="5" t="n">
+      <c r="L232" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M232" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N232" s="5" t="n">
         <v>5.3</v>
       </c>
-      <c r="O231" s="5" t="n">
+      <c r="O232" s="5" t="n">
         <v>18</v>
       </c>
     </row>
-    <row r="232" ht="58" customHeight="1">
-      <c r="A232" s="9">
+    <row r="233" ht="58" customHeight="1">
+      <c r="A233" s="9">
         <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
         <v/>
       </c>
-      <c r="B232" s="10" t="inlineStr">
+      <c r="B233" s="10" t="inlineStr">
         <is>
           <t>Listmonk</t>
         </is>
       </c>
-      <c r="C232" s="11" t="inlineStr">
+      <c r="C233" s="11" t="inlineStr">
         <is>
           <t>Open source (GitHub)</t>
         </is>
       </c>
-      <c r="D232" s="12" t="inlineStr">
+      <c r="D233" s="12" t="inlineStr">
         <is>
           <t>github.com/knadh/listmonk</t>
         </is>
       </c>
-      <c r="E232" s="11" t="inlineStr">
+      <c r="E233" s="11" t="inlineStr">
         <is>
           <t>Self-hosted high-performance email campaign and newsletter manager</t>
         </is>
       </c>
-      <c r="F232" s="11" t="inlineStr">
+      <c r="F233" s="11" t="inlineStr">
         <is>
           <t>Free (self-host)</t>
         </is>
       </c>
-      <c r="G232" s="11" t="inlineStr">
+      <c r="G233" s="11" t="inlineStr">
         <is>
           <t>Partial — pair with Claude to draft campaigns</t>
         </is>
       </c>
-      <c r="H232" s="11" t="inlineStr">
+      <c r="H233" s="11" t="inlineStr">
         <is>
           <t>Free at any scale; fast; API-driven</t>
         </is>
       </c>
-      <c r="I232" s="11" t="inlineStr">
+      <c r="I233" s="11" t="inlineStr">
         <is>
           <t>Warm-list campaigns, not cold outreach</t>
         </is>
       </c>
-      <c r="J232" s="11" t="inlineStr">
+      <c r="J233" s="11" t="inlineStr">
         <is>
           <t>Self-hosters sending email campaigns</t>
         </is>
       </c>
-      <c r="K232" s="9" t="n">
+      <c r="K233" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="L232" s="9" t="n">
+      <c r="L233" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="M232" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N232" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="O232" s="9" t="n">
+      <c r="M233" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N233" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="O233" s="9" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="233" ht="22" customHeight="1">
-      <c r="A233" s="4" t="inlineStr">
+    <row r="234" ht="22" customHeight="1">
+      <c r="A234" s="4" t="inlineStr">
         <is>
           <t>AI Marketing &amp; SEO</t>
         </is>
-      </c>
-    </row>
-    <row r="234" ht="58" customHeight="1">
-      <c r="A234" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=semrush.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B234" s="6" t="inlineStr">
-        <is>
-          <t>Semrush</t>
-        </is>
-      </c>
-      <c r="C234" s="7" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="D234" s="8" t="inlineStr">
-        <is>
-          <t>semrush.com</t>
-        </is>
-      </c>
-      <c r="E234" s="7" t="inlineStr">
-        <is>
-          <t>All-in-one SEO/SEM platform with AI features and ContentShake</t>
-        </is>
-      </c>
-      <c r="F234" s="7" t="inlineStr">
-        <is>
-          <t>From $139.95/mo</t>
-        </is>
-      </c>
-      <c r="G234" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H234" s="7" t="inlineStr">
-        <is>
-          <t>Deepest SEO dataset; AI content tools</t>
-        </is>
-      </c>
-      <c r="I234" s="7" t="inlineStr">
-        <is>
-          <t>Expensive; overwhelming</t>
-        </is>
-      </c>
-      <c r="J234" s="7" t="inlineStr">
-        <is>
-          <t>SEO professionals</t>
-        </is>
-      </c>
-      <c r="K234" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="L234" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="M234" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="N234" s="5" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="O234" s="5" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="235" ht="58" customHeight="1">
       <c r="A235" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=ahrefs.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=semrush.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B235" s="6" t="inlineStr">
         <is>
-          <t>Ahrefs</t>
+          <t>Semrush</t>
         </is>
       </c>
       <c r="C235" s="7" t="inlineStr">
@@ -15109,17 +15109,17 @@
       </c>
       <c r="D235" s="8" t="inlineStr">
         <is>
-          <t>ahrefs.com</t>
+          <t>semrush.com</t>
         </is>
       </c>
       <c r="E235" s="7" t="inlineStr">
         <is>
-          <t>Backlink/keyword research leader with AI content helper</t>
+          <t>All-in-one SEO/SEM platform with AI features and ContentShake</t>
         </is>
       </c>
       <c r="F235" s="7" t="inlineStr">
         <is>
-          <t>From $129/mo</t>
+          <t>From $139.95/mo</t>
         </is>
       </c>
       <c r="G235" s="7" t="inlineStr">
@@ -15129,21 +15129,21 @@
       </c>
       <c r="H235" s="7" t="inlineStr">
         <is>
-          <t>Best link data; clean UX</t>
+          <t>Deepest SEO dataset; AI content tools</t>
         </is>
       </c>
       <c r="I235" s="7" t="inlineStr">
         <is>
-          <t>No free tier; AI is light</t>
+          <t>Expensive; overwhelming</t>
         </is>
       </c>
       <c r="J235" s="7" t="inlineStr">
         <is>
-          <t>Link-building and SEO research</t>
+          <t>SEO professionals</t>
         </is>
       </c>
       <c r="K235" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L235" s="5" t="n">
         <v>4</v>
@@ -15152,20 +15152,20 @@
         <v>9</v>
       </c>
       <c r="N235" s="5" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="O235" s="5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="236" ht="58" customHeight="1">
       <c r="A236" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=surferseo.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=ahrefs.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B236" s="6" t="inlineStr">
         <is>
-          <t>Surfer</t>
+          <t>Ahrefs</t>
         </is>
       </c>
       <c r="C236" s="7" t="inlineStr">
@@ -15175,17 +15175,17 @@
       </c>
       <c r="D236" s="8" t="inlineStr">
         <is>
-          <t>surferseo.com</t>
+          <t>ahrefs.com</t>
         </is>
       </c>
       <c r="E236" s="7" t="inlineStr">
         <is>
-          <t>On-page SEO content optimisation with AI writing</t>
+          <t>Backlink/keyword research leader with AI content helper</t>
         </is>
       </c>
       <c r="F236" s="7" t="inlineStr">
         <is>
-          <t>From $89/mo</t>
+          <t>From $129/mo</t>
         </is>
       </c>
       <c r="G236" s="7" t="inlineStr">
@@ -15195,43 +15195,43 @@
       </c>
       <c r="H236" s="7" t="inlineStr">
         <is>
-          <t>Clear data-driven content scores</t>
+          <t>Best link data; clean UX</t>
         </is>
       </c>
       <c r="I236" s="7" t="inlineStr">
         <is>
-          <t>Per-article economics; SERP-chasing risk</t>
+          <t>No free tier; AI is light</t>
         </is>
       </c>
       <c r="J236" s="7" t="inlineStr">
         <is>
-          <t>Content teams optimising for Google</t>
+          <t>Link-building and SEO research</t>
         </is>
       </c>
       <c r="K236" s="5" t="n">
         <v>5</v>
       </c>
       <c r="L236" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M236" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N236" s="5" t="n">
         <v>6</v>
       </c>
       <c r="O236" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="237" ht="58" customHeight="1">
       <c r="A237" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=adcreative.ai&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=surferseo.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B237" s="6" t="inlineStr">
         <is>
-          <t>AdCreative.ai</t>
+          <t>Surfer</t>
         </is>
       </c>
       <c r="C237" s="7" t="inlineStr">
@@ -15241,17 +15241,17 @@
       </c>
       <c r="D237" s="8" t="inlineStr">
         <is>
-          <t>adcreative.ai</t>
+          <t>surferseo.com</t>
         </is>
       </c>
       <c r="E237" s="7" t="inlineStr">
         <is>
-          <t>AI ad creative and copy generation with performance scoring</t>
+          <t>On-page SEO content optimisation with AI writing</t>
         </is>
       </c>
       <c r="F237" s="7" t="inlineStr">
         <is>
-          <t>From $25/mo</t>
+          <t>From $89/mo</t>
         </is>
       </c>
       <c r="G237" s="7" t="inlineStr">
@@ -15261,43 +15261,43 @@
       </c>
       <c r="H237" s="7" t="inlineStr">
         <is>
-          <t>Volume ad-variant generation; scoring</t>
+          <t>Clear data-driven content scores</t>
         </is>
       </c>
       <c r="I237" s="7" t="inlineStr">
         <is>
-          <t>Template look; aggressive billing reputation — check terms</t>
+          <t>Per-article economics; SERP-chasing risk</t>
         </is>
       </c>
       <c r="J237" s="7" t="inlineStr">
         <is>
-          <t>Performance marketers</t>
+          <t>Content teams optimising for Google</t>
         </is>
       </c>
       <c r="K237" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L237" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M237" s="5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N237" s="5" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
       <c r="O237" s="5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="238" ht="58" customHeight="1">
       <c r="A238" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=hootsuite.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=adcreative.ai&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B238" s="6" t="inlineStr">
         <is>
-          <t>Hootsuite</t>
+          <t>AdCreative.ai</t>
         </is>
       </c>
       <c r="C238" s="7" t="inlineStr">
@@ -15307,17 +15307,17 @@
       </c>
       <c r="D238" s="8" t="inlineStr">
         <is>
-          <t>hootsuite.com</t>
+          <t>adcreative.ai</t>
         </is>
       </c>
       <c r="E238" s="7" t="inlineStr">
         <is>
-          <t>Social media management with OwlyWriter AI</t>
+          <t>AI ad creative and copy generation with performance scoring</t>
         </is>
       </c>
       <c r="F238" s="7" t="inlineStr">
         <is>
-          <t>From $99/mo</t>
+          <t>From $25/mo</t>
         </is>
       </c>
       <c r="G238" s="7" t="inlineStr">
@@ -15327,63 +15327,63 @@
       </c>
       <c r="H238" s="7" t="inlineStr">
         <is>
-          <t>Mature scheduling/listening suite</t>
+          <t>Volume ad-variant generation; scoring</t>
         </is>
       </c>
       <c r="I238" s="7" t="inlineStr">
         <is>
-          <t>Expensive; AI basic</t>
+          <t>Template look; aggressive billing reputation — check terms</t>
         </is>
       </c>
       <c r="J238" s="7" t="inlineStr">
         <is>
-          <t>Social teams managing many accounts</t>
+          <t>Performance marketers</t>
         </is>
       </c>
       <c r="K238" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L238" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M238" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N238" s="5" t="n">
         <v>5.3</v>
       </c>
       <c r="O238" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="239" ht="58" customHeight="1">
       <c r="A239" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=buffer.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=hootsuite.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B239" s="6" t="inlineStr">
         <is>
-          <t>Buffer</t>
+          <t>Hootsuite</t>
         </is>
       </c>
       <c r="C239" s="7" t="inlineStr">
         <is>
-          <t>Freemium</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="D239" s="8" t="inlineStr">
         <is>
-          <t>buffer.com</t>
+          <t>hootsuite.com</t>
         </is>
       </c>
       <c r="E239" s="7" t="inlineStr">
         <is>
-          <t>Simple social scheduling with AI assistant</t>
+          <t>Social media management with OwlyWriter AI</t>
         </is>
       </c>
       <c r="F239" s="7" t="inlineStr">
         <is>
-          <t>Free; $6/channel/mo</t>
+          <t>From $99/mo</t>
         </is>
       </c>
       <c r="G239" s="7" t="inlineStr">
@@ -15393,43 +15393,43 @@
       </c>
       <c r="H239" s="7" t="inlineStr">
         <is>
-          <t>Affordable; clean; good AI repurposing</t>
+          <t>Mature scheduling/listening suite</t>
         </is>
       </c>
       <c r="I239" s="7" t="inlineStr">
         <is>
-          <t>Lighter analytics</t>
+          <t>Expensive; AI basic</t>
         </is>
       </c>
       <c r="J239" s="7" t="inlineStr">
         <is>
-          <t>Creators and small brands</t>
+          <t>Social teams managing many accounts</t>
         </is>
       </c>
       <c r="K239" s="5" t="n">
         <v>5</v>
       </c>
       <c r="L239" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M239" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N239" s="5" t="n">
-        <v>6.3</v>
+        <v>5.3</v>
       </c>
       <c r="O239" s="5" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="240" ht="58" customHeight="1">
       <c r="A240" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=mailchimp.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=buffer.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B240" s="6" t="inlineStr">
         <is>
-          <t>Mailchimp</t>
+          <t>Buffer</t>
         </is>
       </c>
       <c r="C240" s="7" t="inlineStr">
@@ -15439,17 +15439,17 @@
       </c>
       <c r="D240" s="8" t="inlineStr">
         <is>
-          <t>mailchimp.com</t>
+          <t>buffer.com</t>
         </is>
       </c>
       <c r="E240" s="7" t="inlineStr">
         <is>
-          <t>Email marketing with AI content and journeys</t>
+          <t>Simple social scheduling with AI assistant</t>
         </is>
       </c>
       <c r="F240" s="7" t="inlineStr">
         <is>
-          <t>Free; from $13/mo</t>
+          <t>Free; $6/channel/mo</t>
         </is>
       </c>
       <c r="G240" s="7" t="inlineStr">
@@ -15459,165 +15459,165 @@
       </c>
       <c r="H240" s="7" t="inlineStr">
         <is>
-          <t>Familiar; AI campaign generation</t>
+          <t>Affordable; clean; good AI repurposing</t>
         </is>
       </c>
       <c r="I240" s="7" t="inlineStr">
         <is>
-          <t>Pricing grows with list; CRM-lite</t>
+          <t>Lighter analytics</t>
         </is>
       </c>
       <c r="J240" s="7" t="inlineStr">
         <is>
-          <t>SMB email marketing</t>
+          <t>Creators and small brands</t>
         </is>
       </c>
       <c r="K240" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L240" s="5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M240" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N240" s="5" t="n">
         <v>6.3</v>
       </c>
       <c r="O240" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="241" ht="58" customHeight="1">
       <c r="A241" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=mailchimp.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B241" s="6" t="inlineStr">
+        <is>
+          <t>Mailchimp</t>
+        </is>
+      </c>
+      <c r="C241" s="7" t="inlineStr">
+        <is>
+          <t>Freemium</t>
+        </is>
+      </c>
+      <c r="D241" s="8" t="inlineStr">
+        <is>
+          <t>mailchimp.com</t>
+        </is>
+      </c>
+      <c r="E241" s="7" t="inlineStr">
+        <is>
+          <t>Email marketing with AI content and journeys</t>
+        </is>
+      </c>
+      <c r="F241" s="7" t="inlineStr">
+        <is>
+          <t>Free; from $13/mo</t>
+        </is>
+      </c>
+      <c r="G241" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H241" s="7" t="inlineStr">
+        <is>
+          <t>Familiar; AI campaign generation</t>
+        </is>
+      </c>
+      <c r="I241" s="7" t="inlineStr">
+        <is>
+          <t>Pricing grows with list; CRM-lite</t>
+        </is>
+      </c>
+      <c r="J241" s="7" t="inlineStr">
+        <is>
+          <t>SMB email marketing</t>
+        </is>
+      </c>
+      <c r="K241" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="L241" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M241" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="N241" s="5" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="O241" s="5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="242" ht="58" customHeight="1">
+      <c r="A242" s="5">
         <f>IMAGE("https://www.google.com/s2/favicons?domain=trysoro.com&amp;sz=64")</f>
         <v/>
       </c>
-      <c r="B241" s="6" t="inlineStr">
+      <c r="B242" s="6" t="inlineStr">
         <is>
           <t>Soro</t>
         </is>
       </c>
-      <c r="C241" s="7" t="inlineStr">
+      <c r="C242" s="7" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
-      <c r="D241" s="8" t="inlineStr">
+      <c r="D242" s="8" t="inlineStr">
         <is>
           <t>trysoro.com</t>
         </is>
       </c>
-      <c r="E241" s="7" t="inlineStr">
+      <c r="E242" s="7" t="inlineStr">
         <is>
           <t>SEO autopilot: researches keywords, writes, optimises and auto-publishes articles (WordPress/Shopify/Webflow)</t>
         </is>
       </c>
-      <c r="F241" s="7" t="inlineStr">
+      <c r="F242" s="7" t="inlineStr">
         <is>
           <t>From $39/mo</t>
         </is>
       </c>
-      <c r="G241" s="7" t="inlineStr">
+      <c r="G242" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H241" s="7" t="inlineStr">
+      <c r="H242" s="7" t="inlineStr">
         <is>
           <t>Hands-off SEO content pipeline; cheap</t>
         </is>
       </c>
-      <c r="I241" s="7" t="inlineStr">
+      <c r="I242" s="7" t="inlineStr">
         <is>
           <t>AI-content quality and Google-policy risk need human review</t>
         </is>
       </c>
-      <c r="J241" s="7" t="inlineStr">
+      <c r="J242" s="7" t="inlineStr">
         <is>
           <t>Niche-site builders and small ecommerce</t>
         </is>
       </c>
-      <c r="K241" s="5" t="n">
+      <c r="K242" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="L241" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="M241" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="N241" s="5" t="n">
+      <c r="L242" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="M242" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N242" s="5" t="n">
         <v>5.7</v>
       </c>
-      <c r="O241" s="5" t="n">
+      <c r="O242" s="5" t="n">
         <v>9</v>
-      </c>
-    </row>
-    <row r="242" ht="58" customHeight="1">
-      <c r="A242" s="9">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B242" s="10" t="inlineStr">
-        <is>
-          <t>Mautic</t>
-        </is>
-      </c>
-      <c r="C242" s="11" t="inlineStr">
-        <is>
-          <t>Open source (GitHub)</t>
-        </is>
-      </c>
-      <c r="D242" s="12" t="inlineStr">
-        <is>
-          <t>github.com/mautic/mautic</t>
-        </is>
-      </c>
-      <c r="E242" s="11" t="inlineStr">
-        <is>
-          <t>Open-source marketing automation (email, journeys, segmentation)</t>
-        </is>
-      </c>
-      <c r="F242" s="11" t="inlineStr">
-        <is>
-          <t>Free (self-host)</t>
-        </is>
-      </c>
-      <c r="G242" s="11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H242" s="11" t="inlineStr">
-        <is>
-          <t>Full marketing automation without per-contact fees</t>
-        </is>
-      </c>
-      <c r="I242" s="11" t="inlineStr">
-        <is>
-          <t>Self-host complexity; plugins needed</t>
-        </is>
-      </c>
-      <c r="J242" s="11" t="inlineStr">
-        <is>
-          <t>Companies escaping HubSpot/Marketo pricing</t>
-        </is>
-      </c>
-      <c r="K242" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="L242" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="M242" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="N242" s="9" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="O242" s="9" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="243" ht="58" customHeight="1">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B243" s="10" t="inlineStr">
         <is>
-          <t>Postiz</t>
+          <t>Mautic</t>
         </is>
       </c>
       <c r="C243" s="11" t="inlineStr">
@@ -15637,53 +15637,53 @@
       </c>
       <c r="D243" s="12" t="inlineStr">
         <is>
-          <t>github.com/gitroomhq/postiz-app</t>
+          <t>github.com/mautic/mautic</t>
         </is>
       </c>
       <c r="E243" s="11" t="inlineStr">
         <is>
-          <t>Open-source AI social media scheduling (Buffer/Hootsuite alternative)</t>
+          <t>Open-source marketing automation (email, journeys, segmentation)</t>
         </is>
       </c>
       <c r="F243" s="11" t="inlineStr">
         <is>
-          <t>Free self-host; cloud from $29/mo</t>
+          <t>Free (self-host)</t>
         </is>
       </c>
       <c r="G243" s="11" t="inlineStr">
         <is>
-          <t>Partial — BYO AI keys</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H243" s="11" t="inlineStr">
         <is>
-          <t>OSS scheduling for 15+ platforms with AI</t>
+          <t>Full marketing automation without per-contact fees</t>
         </is>
       </c>
       <c r="I243" s="11" t="inlineStr">
         <is>
-          <t>Young project</t>
+          <t>Self-host complexity; plugins needed</t>
         </is>
       </c>
       <c r="J243" s="11" t="inlineStr">
         <is>
-          <t>Self-hosted social scheduling</t>
+          <t>Companies escaping HubSpot/Marketo pricing</t>
         </is>
       </c>
       <c r="K243" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L243" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M243" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N243" s="9" t="n">
-        <v>7</v>
+        <v>7.3</v>
       </c>
       <c r="O243" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="244" ht="58" customHeight="1">
@@ -15693,7 +15693,7 @@
       </c>
       <c r="B244" s="10" t="inlineStr">
         <is>
-          <t>Matomo</t>
+          <t>Postiz</t>
         </is>
       </c>
       <c r="C244" s="11" t="inlineStr">
@@ -15703,136 +15703,136 @@
       </c>
       <c r="D244" s="12" t="inlineStr">
         <is>
-          <t>github.com/matomo-org/matomo</t>
+          <t>github.com/gitroomhq/postiz-app</t>
         </is>
       </c>
       <c r="E244" s="11" t="inlineStr">
         <is>
-          <t>Open-source web analytics (Google Analytics alternative)</t>
+          <t>Open-source AI social media scheduling (Buffer/Hootsuite alternative)</t>
         </is>
       </c>
       <c r="F244" s="11" t="inlineStr">
         <is>
-          <t>Free self-host; cloud from $23/mo</t>
+          <t>Free self-host; cloud from $29/mo</t>
         </is>
       </c>
       <c r="G244" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partial — BYO AI keys</t>
         </is>
       </c>
       <c r="H244" s="11" t="inlineStr">
         <is>
-          <t>Privacy-compliant analytics you own</t>
+          <t>OSS scheduling for 15+ platforms with AI</t>
         </is>
       </c>
       <c r="I244" s="11" t="inlineStr">
         <is>
-          <t>No AI insights layer yet</t>
+          <t>Young project</t>
         </is>
       </c>
       <c r="J244" s="11" t="inlineStr">
         <is>
-          <t>Privacy-first site analytics</t>
+          <t>Self-hosted social scheduling</t>
         </is>
       </c>
       <c r="K244" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L244" s="9" t="n">
         <v>9</v>
       </c>
       <c r="M244" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N244" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="O244" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="245" ht="58" customHeight="1">
+      <c r="A245" s="9">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B245" s="10" t="inlineStr">
+        <is>
+          <t>Matomo</t>
+        </is>
+      </c>
+      <c r="C245" s="11" t="inlineStr">
+        <is>
+          <t>Open source (GitHub)</t>
+        </is>
+      </c>
+      <c r="D245" s="12" t="inlineStr">
+        <is>
+          <t>github.com/matomo-org/matomo</t>
+        </is>
+      </c>
+      <c r="E245" s="11" t="inlineStr">
+        <is>
+          <t>Open-source web analytics (Google Analytics alternative)</t>
+        </is>
+      </c>
+      <c r="F245" s="11" t="inlineStr">
+        <is>
+          <t>Free self-host; cloud from $23/mo</t>
+        </is>
+      </c>
+      <c r="G245" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H245" s="11" t="inlineStr">
+        <is>
+          <t>Privacy-compliant analytics you own</t>
+        </is>
+      </c>
+      <c r="I245" s="11" t="inlineStr">
+        <is>
+          <t>No AI insights layer yet</t>
+        </is>
+      </c>
+      <c r="J245" s="11" t="inlineStr">
+        <is>
+          <t>Privacy-first site analytics</t>
+        </is>
+      </c>
+      <c r="K245" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L245" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="M245" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="N245" s="9" t="n">
         <v>6.7</v>
       </c>
-      <c r="O244" s="9" t="n">
+      <c r="O245" s="9" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="245" ht="22" customHeight="1">
-      <c r="A245" s="4" t="inlineStr">
+    <row r="246" ht="22" customHeight="1">
+      <c r="A246" s="4" t="inlineStr">
         <is>
           <t>AI Research Tools</t>
         </is>
-      </c>
-    </row>
-    <row r="246" ht="58" customHeight="1">
-      <c r="A246" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=elicit.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B246" s="6" t="inlineStr">
-        <is>
-          <t>Elicit</t>
-        </is>
-      </c>
-      <c r="C246" s="7" t="inlineStr">
-        <is>
-          <t>Freemium</t>
-        </is>
-      </c>
-      <c r="D246" s="8" t="inlineStr">
-        <is>
-          <t>elicit.com</t>
-        </is>
-      </c>
-      <c r="E246" s="7" t="inlineStr">
-        <is>
-          <t>AI research assistant that searches and summarises academic papers</t>
-        </is>
-      </c>
-      <c r="F246" s="7" t="inlineStr">
-        <is>
-          <t>Free; Plus $12/mo</t>
-        </is>
-      </c>
-      <c r="G246" s="7" t="inlineStr">
-        <is>
-          <t>No — (Anthropic models used under the hood historically)</t>
-        </is>
-      </c>
-      <c r="H246" s="7" t="inlineStr">
-        <is>
-          <t>Systematic-review-grade extraction tables</t>
-        </is>
-      </c>
-      <c r="I246" s="7" t="inlineStr">
-        <is>
-          <t>Academic papers only</t>
-        </is>
-      </c>
-      <c r="J246" s="7" t="inlineStr">
-        <is>
-          <t>Researchers and grad students</t>
-        </is>
-      </c>
-      <c r="K246" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="L246" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="M246" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="N246" s="5" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="O246" s="5" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="247" ht="58" customHeight="1">
       <c r="A247" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=consensus.app&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=elicit.com&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B247" s="6" t="inlineStr">
         <is>
-          <t>Consensus</t>
+          <t>Elicit</t>
         </is>
       </c>
       <c r="C247" s="7" t="inlineStr">
@@ -15842,63 +15842,63 @@
       </c>
       <c r="D247" s="8" t="inlineStr">
         <is>
-          <t>consensus.app</t>
+          <t>elicit.com</t>
         </is>
       </c>
       <c r="E247" s="7" t="inlineStr">
         <is>
-          <t>Search engine answering questions from peer-reviewed evidence</t>
+          <t>AI research assistant that searches and summarises academic papers</t>
         </is>
       </c>
       <c r="F247" s="7" t="inlineStr">
         <is>
-          <t>Free; Premium $11.99/mo</t>
+          <t>Free; Plus $12/mo</t>
         </is>
       </c>
       <c r="G247" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No — (Anthropic models used under the hood historically)</t>
         </is>
       </c>
       <c r="H247" s="7" t="inlineStr">
         <is>
-          <t>Evidence meters; citation-grounded answers</t>
+          <t>Systematic-review-grade extraction tables</t>
         </is>
       </c>
       <c r="I247" s="7" t="inlineStr">
         <is>
-          <t>Narrower than general search</t>
+          <t>Academic papers only</t>
         </is>
       </c>
       <c r="J247" s="7" t="inlineStr">
         <is>
-          <t>Evidence-based professionals</t>
+          <t>Researchers and grad students</t>
         </is>
       </c>
       <c r="K247" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L247" s="5" t="n">
         <v>7</v>
       </c>
       <c r="M247" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N247" s="5" t="n">
-        <v>6</v>
+        <v>6.7</v>
       </c>
       <c r="O247" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="248" ht="58" customHeight="1">
       <c r="A248" s="5">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=scispace.com&amp;sz=64")</f>
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=consensus.app&amp;sz=64")</f>
         <v/>
       </c>
       <c r="B248" s="6" t="inlineStr">
         <is>
-          <t>SciSpace</t>
+          <t>Consensus</t>
         </is>
       </c>
       <c r="C248" s="7" t="inlineStr">
@@ -15908,17 +15908,17 @@
       </c>
       <c r="D248" s="8" t="inlineStr">
         <is>
-          <t>scispace.com</t>
+          <t>consensus.app</t>
         </is>
       </c>
       <c r="E248" s="7" t="inlineStr">
         <is>
-          <t>Read, annotate and chat with research PDFs; literature review AI</t>
+          <t>Search engine answering questions from peer-reviewed evidence</t>
         </is>
       </c>
       <c r="F248" s="7" t="inlineStr">
         <is>
-          <t>Free; from $12/mo</t>
+          <t>Free; Premium $11.99/mo</t>
         </is>
       </c>
       <c r="G248" s="7" t="inlineStr">
@@ -15928,17 +15928,17 @@
       </c>
       <c r="H248" s="7" t="inlineStr">
         <is>
-          <t>Great PDF explanation UX</t>
+          <t>Evidence meters; citation-grounded answers</t>
         </is>
       </c>
       <c r="I248" s="7" t="inlineStr">
         <is>
-          <t>Aggressive upsells</t>
+          <t>Narrower than general search</t>
         </is>
       </c>
       <c r="J248" s="7" t="inlineStr">
         <is>
-          <t>Students decoding dense papers</t>
+          <t>Evidence-based professionals</t>
         </is>
       </c>
       <c r="K248" s="5" t="n">
@@ -15948,79 +15948,79 @@
         <v>7</v>
       </c>
       <c r="M248" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N248" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="O248" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="249" ht="58" customHeight="1">
+      <c r="A249" s="5">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=scispace.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B249" s="6" t="inlineStr">
+        <is>
+          <t>SciSpace</t>
+        </is>
+      </c>
+      <c r="C249" s="7" t="inlineStr">
+        <is>
+          <t>Freemium</t>
+        </is>
+      </c>
+      <c r="D249" s="8" t="inlineStr">
+        <is>
+          <t>scispace.com</t>
+        </is>
+      </c>
+      <c r="E249" s="7" t="inlineStr">
+        <is>
+          <t>Read, annotate and chat with research PDFs; literature review AI</t>
+        </is>
+      </c>
+      <c r="F249" s="7" t="inlineStr">
+        <is>
+          <t>Free; from $12/mo</t>
+        </is>
+      </c>
+      <c r="G249" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H249" s="7" t="inlineStr">
+        <is>
+          <t>Great PDF explanation UX</t>
+        </is>
+      </c>
+      <c r="I249" s="7" t="inlineStr">
+        <is>
+          <t>Aggressive upsells</t>
+        </is>
+      </c>
+      <c r="J249" s="7" t="inlineStr">
+        <is>
+          <t>Students decoding dense papers</t>
+        </is>
+      </c>
+      <c r="K249" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L249" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="M249" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="N249" s="5" t="n">
         <v>5.7</v>
       </c>
-      <c r="O248" s="5" t="n">
+      <c r="O249" s="5" t="n">
         <v>5</v>
-      </c>
-    </row>
-    <row r="249" ht="58" customHeight="1">
-      <c r="A249" s="9">
-        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
-        <v/>
-      </c>
-      <c r="B249" s="10" t="inlineStr">
-        <is>
-          <t>GPT Researcher</t>
-        </is>
-      </c>
-      <c r="C249" s="11" t="inlineStr">
-        <is>
-          <t>Open source (GitHub)</t>
-        </is>
-      </c>
-      <c r="D249" s="12" t="inlineStr">
-        <is>
-          <t>github.com/assafelovic/gpt-researcher</t>
-        </is>
-      </c>
-      <c r="E249" s="11" t="inlineStr">
-        <is>
-          <t>Open-source autonomous deep-research agent producing cited reports</t>
-        </is>
-      </c>
-      <c r="F249" s="11" t="inlineStr">
-        <is>
-          <t>Free + API costs</t>
-        </is>
-      </c>
-      <c r="G249" s="11" t="inlineStr">
-        <is>
-          <t>Yes — supports Anthropic/Claude as the LLM</t>
-        </is>
-      </c>
-      <c r="H249" s="11" t="inlineStr">
-        <is>
-          <t>Free deep-research with citations; local &amp; web</t>
-        </is>
-      </c>
-      <c r="I249" s="11" t="inlineStr">
-        <is>
-          <t>Setup + API keys; report quality varies by model</t>
-        </is>
-      </c>
-      <c r="J249" s="11" t="inlineStr">
-        <is>
-          <t>Developers automating research</t>
-        </is>
-      </c>
-      <c r="K249" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="L249" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="M249" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="N249" s="9" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="O249" s="9" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="250" ht="58" customHeight="1">
@@ -16030,7 +16030,7 @@
       </c>
       <c r="B250" s="10" t="inlineStr">
         <is>
-          <t>STORM</t>
+          <t>GPT Researcher</t>
         </is>
       </c>
       <c r="C250" s="11" t="inlineStr">
@@ -16040,12 +16040,12 @@
       </c>
       <c r="D250" s="12" t="inlineStr">
         <is>
-          <t>github.com/stanford-oval/storm</t>
+          <t>github.com/assafelovic/gpt-researcher</t>
         </is>
       </c>
       <c r="E250" s="11" t="inlineStr">
         <is>
-          <t>Stanford's open-source Wikipedia-style article research/writing system</t>
+          <t>Open-source autonomous deep-research agent producing cited reports</t>
         </is>
       </c>
       <c r="F250" s="11" t="inlineStr">
@@ -16055,59 +16055,125 @@
       </c>
       <c r="G250" s="11" t="inlineStr">
         <is>
-          <t>Yes — configurable to Claude models</t>
+          <t>Yes — supports Anthropic/Claude as the LLM</t>
         </is>
       </c>
       <c r="H250" s="11" t="inlineStr">
         <is>
-          <t>Research-grade outline→article pipeline</t>
+          <t>Free deep-research with citations; local &amp; web</t>
         </is>
       </c>
       <c r="I250" s="11" t="inlineStr">
         <is>
-          <t>Academic tool; rough edges</t>
+          <t>Setup + API keys; report quality varies by model</t>
         </is>
       </c>
       <c r="J250" s="11" t="inlineStr">
         <is>
-          <t>Long-form grounded content experiments</t>
+          <t>Developers automating research</t>
         </is>
       </c>
       <c r="K250" s="9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L250" s="9" t="n">
         <v>9</v>
       </c>
       <c r="M250" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N250" s="9" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="O250" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="251" ht="58" customHeight="1">
+      <c r="A251" s="9">
+        <f>IMAGE("https://www.google.com/s2/favicons?domain=github.com&amp;sz=64")</f>
+        <v/>
+      </c>
+      <c r="B251" s="10" t="inlineStr">
+        <is>
+          <t>STORM</t>
+        </is>
+      </c>
+      <c r="C251" s="11" t="inlineStr">
+        <is>
+          <t>Open source (GitHub)</t>
+        </is>
+      </c>
+      <c r="D251" s="12" t="inlineStr">
+        <is>
+          <t>github.com/stanford-oval/storm</t>
+        </is>
+      </c>
+      <c r="E251" s="11" t="inlineStr">
+        <is>
+          <t>Stanford's open-source Wikipedia-style article research/writing system</t>
+        </is>
+      </c>
+      <c r="F251" s="11" t="inlineStr">
+        <is>
+          <t>Free + API costs</t>
+        </is>
+      </c>
+      <c r="G251" s="11" t="inlineStr">
+        <is>
+          <t>Yes — configurable to Claude models</t>
+        </is>
+      </c>
+      <c r="H251" s="11" t="inlineStr">
+        <is>
+          <t>Research-grade outline→article pipeline</t>
+        </is>
+      </c>
+      <c r="I251" s="11" t="inlineStr">
+        <is>
+          <t>Academic tool; rough edges</t>
+        </is>
+      </c>
+      <c r="J251" s="11" t="inlineStr">
+        <is>
+          <t>Long-form grounded content experiments</t>
+        </is>
+      </c>
+      <c r="K251" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="L251" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="M251" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N251" s="9" t="n">
         <v>6.7</v>
       </c>
-      <c r="O250" s="9" t="n">
+      <c r="O251" s="9" t="n">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A233:O233"/>
     <mergeCell ref="A46:O46"/>
+    <mergeCell ref="A208:O208"/>
+    <mergeCell ref="A246:O246"/>
     <mergeCell ref="A101:O101"/>
     <mergeCell ref="A136:O136"/>
     <mergeCell ref="A154:O154"/>
     <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A234:O234"/>
     <mergeCell ref="A144:O144"/>
     <mergeCell ref="A122:O122"/>
     <mergeCell ref="A165:O165"/>
     <mergeCell ref="A112:O112"/>
     <mergeCell ref="A34:O34"/>
-    <mergeCell ref="A245:O245"/>
     <mergeCell ref="A176:O176"/>
     <mergeCell ref="A15:O15"/>
     <mergeCell ref="A59:O59"/>
     <mergeCell ref="A191:O191"/>
-    <mergeCell ref="A207:O207"/>
     <mergeCell ref="A88:O88"/>
     <mergeCell ref="A78:O78"/>
   </mergeCells>
@@ -16301,7 +16367,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D204" r:id="rId187"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D205" r:id="rId188"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D206" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D208" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D207" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D209" r:id="rId191"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D210" r:id="rId192"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId193"/>
@@ -16326,7 +16392,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D230" r:id="rId212"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D231" r:id="rId213"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D232" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D234" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D233" r:id="rId215"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D235" r:id="rId216"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D236" r:id="rId217"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D237" r:id="rId218"/>
@@ -16337,11 +16403,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D242" r:id="rId223"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D243" r:id="rId224"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D244" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D246" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D245" r:id="rId226"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D247" r:id="rId227"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D248" r:id="rId228"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D249" r:id="rId229"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D250" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D251" r:id="rId231"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>